<commit_message>
fix permission issue final
</commit_message>
<xml_diff>
--- a/legasus/backend/data/banners.xlsx
+++ b/legasus/backend/data/banners.xlsx
@@ -397,10 +397,67 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:D4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>department</v>
+      </c>
+      <c r="C1" t="str">
+        <v>image</v>
+      </c>
+      <c r="D1" t="str">
+        <v>createdAt</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>banner-men-1775191934086-0</v>
+      </c>
+      <c r="B2" t="str">
+        <v>men</v>
+      </c>
+      <c r="C2" t="str">
+        <v>data:image/webp;base64,UklGRi5RAABXRUJQVlA4WAoAAAAgAAAAAgMAuwIASUNDUMgBAAAAAAHIAAAAAAQwAABtbnRyUkdCIFhZWiAH4AABAAEAAAAAAABhY3NwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAQAA9tYAAQAAAADTLQAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAlkZXNjAAAA8AAAACRyWFlaAAABFAAAABRnWFlaAAABKAAAABRiWFlaAAABPAAAABR3dHB0AAABUAAAABRyVFJDAAABZAAAAChnVFJDAAABZAAAAChiVFJDAAABZAAAAChjcHJ0AAABjAAAADxtbHVjAAAAAAAAAAEAAAAMZW5VUwAAAAgAAAAcAHMAUgBHAEJYWVogAAAAAAAAb6IAADj1AAADkFhZWiAAAAAAAABimQAAt4UAABjaWFlaIAAAAAAAACSgAAAPhAAAts9YWVogAAAAAAAA9tYAAQAAAADTLXBhcmEAAAAAAAQAAAACZmYAAPKnAAANWQAAE9AAAApbAAAAAAAAAABtbHVjAAAAAAAAAAEAAAAMZW5VUwAAACAAAAAcAEcAbwBvAGcAbABlACAASQBuAGMALgAgADIAMAAxADZWUDggQE8AADCnAZ0BKgMDvAI+VSiRRyOiIiEiUNmIcAqJaW77z1mHFfwE285pT8a7+gX0f8B6XHJfiAFfur5ZnQPzAfNH/gesT+5/6n2EeeV5jv2q/aT3UP+h+6Pvf9C7+of4z1mPWS/vf/h9jT9xvTo/bz4ev3Q/b72fP/xrRHo//H/kr4Yf4P+5ft7/ffS38i+ffvH9+/bz+8+3F/beOn1T+j8yP4/9yP0v9q/y3/f/x37sfcv+M/2v+P/Jz1n+QX9J+YH+h+Qj8j/of+Z/v37wf3f1VdtZa7/sf5r2DvbP65/x/8X/of2P9Ov/D/x/rL+gf37/h/4X8nfsC/lX9J/3X+K/JH5m/3Xjt/df+Z7Af9B/xH/S/yH+i/bL6Zf7n/z/6784fed+j/6H/v/5/4Df5x/bf+Z/g+1R6P37qCcj+/aUnw2kZs3Hq3ek4OiiOlixRDR1uujw+aeAzcv6WF652U/SHkkHpEdC+vcx/BaeHdeDZZd4BEyv/cY4ng7QIc/IBgyRwKvoX9SLdmOFAHj9jlo62QE3TrV2TCjxN9GoIStu5dBZc7Bk2BjxPEnvrxxubr8bDXVmM9sTS1cNd1fs1yoXOQ71AMJ3WBqHwnaG9UYJ02xR6GYpv9bUc7OXwqcdq5TTPI/j5fGV937E93Xn6NLh/QnfAHSHx/N7pg3rHQ0FApJl29LaqeB/neC97l5WX752PYoyIH+q6DuvUMzIYyJ9jHJfVqmu7U5c3bqIS3wLN7Gyr4QBxWaNUZ6RfrbaAs9O32dR8CvVKZMRbF38s/USWlr7PUCXxNb+NUXBYvOARSDabsDWa4NbzCivvI5prvsSX4DVrNaTX1l/l9eJmRETd7PikM6iO5I9EdyR6IRzOobvD6zc5W7jGn7L/Mcu3DwvF7BOCKlDmVEdyR5DiIZUR3JHojuSPQ0RDDCO5I9DTyR6GhnVr5fvRW96NxktQP52HtgkuaNW/FXqG+0T2g/cS0GVk9RL1r8znBY8fiP+A0Cm2zOBEaWqp5ylvJIRcnPnQdWvl++dj987H71R5Gu1Qsq44a1i+RW+lHcaQPIG60Ghhw+1tRPc+tUxSnmk61t3plx+vyP9hTKWndvYb/tIlgwp2QPXcxJHcuHSZuo5ckED5yiOrXy/fOx++dj986fAiNgUSZNesPPRngwpjt7SRSyMyAj1MIfpL9goERkjwt/zJiVeSZrPkNbQR8gqdSFeOoCK/LT2QuDrEujEb52P3zsfvnY/fOx7dRWlAmn7raHs9EjHQ5lnm9lyVuhAhL+nnBH6aWigkrXoi95K6epCGJO1LmZ+lSWjWHFHsOW+hwL+gX3zIcfN8PN8r0zN9akt++dj987H752P3zsRVLKEfpXo9EUGyloRzBrDw+g+AsXu3U/Hxiv4jWmQyCDFJK3gu2V7q3Y/fOx++dj987H75bMKcKNitHGWVt4S+C8EpAOwsCb/j85JnAGmsLY7zfR1a+X752P3zsfvnYmQxUHWIpDN7s8NDiwNbuUVg3EVbewmiRJXy/emUJEr752P3zsfvnY/fOx7cRfarQUVdT+wgUWgirSyrd3djTsFKoJrBrcqToOmvKCLJ987H752P3zsfvnYmPdETfy9xhsdMQfyRR7ux/tjsmKOTsKwp6HteD0jZL3gBMZ7Di3TNITQFomi48GTsfvnY/fOx++dj96pXG4JKMG3LXrrgVZUOScC0MWnpwGB7d9jYPmcDCwj2XjxO1+zwmRDtJDjulfHYndokIsa2Yjm2qlssySCVE5Qk3PPRZtactGOEYntfybVFWSOaooulQ2coKULkyP98UsSJ2P3zsfvnY/fOx+ub+1RSV+N2IFXK0cAhCAxepMkF+WJwTdMsy5Aayrg98oYJZyMDRi5vO4ukO67ZIBdJigLeih8r6nkcfIi4dvk7ThoSVBGir/54c1oAEGleMp90mfGU0h5QaWg6tfL987H752P3qqeIsXnMH8P97QsrUJRghCvyuvGSkie/sXwNSQWjVT0KwvMnTAv8EQmUJEr752P3zsfvnY/fOx7cRfarae6gIBAaAMUv1ELtoPttrQjxndKiwTKdq8kV+5rTGuWIWVUHVhpEpjatfL987H752P3zse3EX2q0iNqAkczzJkQnRgjqMnrqsGoSGHEzRknRA0GrDP0wAPei+IUMjv3zpVBhVgtj987H752P3zsfvVNgeq7jxRIo4IQIfPMmQxoBOFPjY/4rMGxEtp3dLPJcNY3h6I61j5b5NbeVZNhw7Hp/tLMRidaCAAaRfvFSokUBhKvyAqWkgVSjOi+1Wvl++dj987HtsMPU/rQeeORoxTw6FeN0QJ5znr+hboowPD1nntidXlVkVKTWi5gXJD0i5EejHtRuyW1zB13QmV/FEbVa+X752P3zsfvnYmT1x5z3WeeG07dPdimsL8WFMkM+epbbjv+JZM8gk1lP/+LS/psMVcQXt3tFORmGBxEAoy+Amr0w+R048lh687a827H752P3zsfvnY/fMQvZvWNN7takUJoHDUyqI5OiJ+vZyjugIo0OsLlVC63LZ5s2b0uS3KIIJtio29Gzk7ZcG74+21v5IvUnoV2P3x/4NX8gSFx6Va+X752P3zsfvnY9uUpgNBd23df8rg5A+yIWSEnFlDOoVxVDv0Mja5EE4JCwwiiMeAm27frHk9zH+aXOGP5sS8yplV4yoHVNtPOi+1Wvl++dj987H66IbFe/8+xynM3pAfwXHfkeG0kBbtUEogwYNROfkDjpKdy361gL0piAZd/+AsZ+g2K1/jcRL+uOivl++dj987H752P3zEZTuwJkDgo9X9SfAYysv0EgtA5Q/HbXU6b2m8JodRnXyE4pggzJo+nSEj2eNxaQCKp4iCps9t8TXy/fOx++dj987H71Vzek6il2gtK/4aTIwPmcT7Ci2ZWOS7cOhczddfk//xmrQyfHBWE0uVbWfij5oLaB1h0stLjpAtzWZp8YePoqyxjfee6g6aJ2P3zsfvnY/fOx+9VdUr6I1Trqrx0376mOs+OntgCLhp286n25JWgPpWiYOaPuGWw9dguh10gfhP7CvnFMbvwWnIMQmhM5mtWGf17XOxfvnY/fOx++dj98xBrdou6do3pBRf6ZnkBJ6cEWw+bOQfD3iC7snsiQeBv93oCtcVa7sLHRPkx8LYo80VtUFTOvaF3mpEQxVYRH2j9LmPvnY/fOx++dj986ansFSQkvP5wOO8Pk7YMPMDPW3MdChbyI9O6fOSEWXo9cx9SiK3v78z4+Hqguuyztkni2I2QGIPZ52ZvyEOX+XY18/b3QdWvl++dj987H75iEoGH6cwMpDodlMdyA5yZ78EguBHd5B7wNvS20Y4p3ccCGQvWftlXOIasiu6pBBsCcuZ6V0QnjUPsOeZvOBTxFi+1Wvl++dj987EyZbwsQO4bxhdpmVwiIWjgEl74eEa03SUFWvq6OxmZ83jygJwn60o3HEe96SMCqbSmI5pyfbcPhNz/0x++dj987H752P3zprqUt0TJGkbGLqMbuhWDuq/sb4YVLUH9w4QovvNdz8aTFE8Dn5qu/5z/kI91e+BPpfZ0XKlyAFMfak3CNIi2P3zsfvnY/fOxMoTJcKRgTtMU79ikWMH4cDN5gnUelqe4YTSA9oMWfhKDPEnYyBllZOKvkD5Ud++dj987H752P3zsTJ7DNPQgSHzqveY8Xqt8AMPi1qejRRs4PthF5zIIgykV5trAP1llNZxgQW8Xi5In0x++dj987H752P3zprqXGNf/ytXMy7DCGEmQFWV88WyNgn3vm9XBHADESYcXn76nEBpxN5SpZfMuT9FsAixfarXy/fOx++dj23F0Mgeo2bP3IslQKYZC6tmIO/0ka+36Uu65lhhqNdSZNL50c/cDNG7DyRwRKUqV8mIEQtlj4h2P5yRi+xC2cxaKMcDcTBuA/UOBIlffOx++dj987H752PbiL8GMQDu4r1OYStyqLHiSycIBC3ohc8YzggKahr7Vay/xSxInY/fOx++dj987H66Cg6tewx/no7fhB8kN0Dzk9Dm4ixfL2lLE1B1a+X752P3zsfvmIozovs424t/maCLF8vaUsTUHVr5fvnY/fOx++X0p4BQn/RfIPT3Zzk5wa3LZlMyV4o/BETsfvnY/fOx++dj18NmDYUrh66SqeRkurUOHKgjdzpbqZZQY8dwUj3cRhCpBZGOmJd66sw+8FoL2CMv5CkT+OPM6WyDWYQ2NK+NYkojhVvliR23auq/AUWRdqMse56yprcgv1tgUBwcwR+ZAysRFsfvnY/fOx++diiz1gUaFN1tbD79tYm7ujeS3tVAJnoUeCFotXg5FxNDCGNNSWPsyqvg70F+CnKnQ6gaPglL5tBBP8YvD3UkdP6JqGRqBm4zGclbVovdi1dOdAUZwXt1DH6oF2P3zsfvnY/fOx++XniYrqfIGoymtsopTNrkZ/p5vXI9EURwx3ksq1C0/++dj987H752P3zse8BvEUgtOj7FLzxPohKujmgNs6tfL987H7zgA/seqfZCYwyjzaPTDbmhfBwIJvU/Ob4YGS5MPK0+xsu5fbFvOUdOcfBhzuSVHwHWsgaUcKOdZOjdyRt+tKtOmpeRtSsB3ft8Gz5ldLusUzmJSxQWnWI3AQWBlQSHzQFf3CGqK4fOAZsKSKI4dxONDuQYpkxpMi8t0RRdw+GGChbDd2+EPkUcVn+bvtGOURgN8hL38F7bL9V63vDT9wbDmzUlf2ZmBnuvjM23tmTGOFMlp5APKgXY7FpCaXNrdXYrDvMWrU6/vt1bqkWmFkEbAw0TFN3Tvid42hNjT3uZ2VjyNMHiocHCdMjem3B03tYEbOImS9vMjjwGwZzv10oOgPTQLYQLokHzuLmsw8+tRwEN4I9efsDYcRZp0dRgGTT+v1MUPBFuULGoGIP0Xwr6/vHikrxXy7eLYX4Pd1lgMJR4coB6AgWfSryDmIOtNdAwemjcOwJv9efFKx/6Pf9J6ZaNhjExSI3or9GKt2CG5bVLrrvg8gx8BgJzW1FUT3kMtd2xQoE37N1I1Rerk7Txy4cOnlYJMeCzIXBsE+84lVN1U1Hbh0q0ngYAi43zouVFE2dDX2ynXE/dcmxlP0QAFN0RVG/zWUQ8D4IK/TRHJvf8joSrcHuOHIAbZ48nG4X6otnIg/GSD5Yp7XMOOnbKr9mtWa9gwXlpvDqIJWNMi+Z7ac6/uzHT68HH+3NMXAf1TCY/D/DzlKRtQcx6qc1wCr02cvccUCneivXg+hLokzpSvy+pgQdRckUyfYDWzMaCn728BJKDR9yclS+9fmfvfs/gXYx95ZMSEa8KZ61K3DqJKVZyLVYWznqrTkVYa9JUpHlanlElgvupSAhgENdCzeO3DQWDLqvIk1YjwaiZpO2HqRv/MozqOyfaFqjH/xN0c6i0A/UPnH/b+Zf6tbxzsR9exY8uZ/qn8Y5qrz2LoW28nL5bKpTQvlIqZ0mUdoDRsv6ujZy0UrEKdryZalEmt59cWmWbwkkMWM+lAwrLC0K8UsX5vZM5fPp31nqt3s66mIMoRgm6ybkGVzP7XXUsK6gVeapI4/ql8/vup9R4j/5jwE7+6bU3FTsj2pXRCWz3ETPfAjvm74l7sAJ5P0UHPojBJ87Xr+VVa44jCjgx5NOq7klQO7mi4I/KNL0MrdQlLRuEYQXdR4/V+L2V47jVil3/8Xdgf/HBvgTh3WiMYf6Zj4tBspaLJgGy/NIB5Rn5RXvDcXDwSUfNeP1j9+pAVeYXdOp27OpftLknIIDAmWBHdJvqwmDSfOfQy1j5dxUP2baLajJeHIw24RvfxF6f5694fvGYTqAuzCrlIiJ+m7yAeeP6p2LJnaO9h1slUW2VCU45xbH0GfOxj8BDSmwMXUsOY2Z5rgF3w52ItKw24goV69dXMJNE4iPqF2nnnFGqvXHatl8joMrOEMRp1MorqkPYI5sYWhqjR/O/tZ9nc9BAJC5hUfm20pp5K+0BpoyXHsCVUPPWff/OxOYBDqAvHHKfdlUM7oit8pcbFM16ukMuOb/LKmEF5Y0heopAOpe+bTDo7GCU5Qi0Cf4j4feIREn8HPq+XH71ZHbGVub2bP9UgfzCsm73TNX4zsxhJTaQOE/QGj3nE7PDHqEGhSMIcjBzCf0NnbT9qs7ouev/6sZqgewcb27ZkG3K+ASctxCNqEhF5cMys9g2TN0foqXJMOECtNDlh9es2rW4CSBnAdaeJ+KPAtPUHrTrl+Jqt12HVIt8hB3xw0uvrzpgci86/x7NCvlSzMCtzOssTHZty2BIHZmFjJSkSOyJGkk8UQ9J8Fhiv0yX9AB+vxnkfsZSCqb5MhR/wXfI1RcjobfzQvb3XCa2bWWWFD4fx4T46NXqzyMZows7nugHCpg6GSb8NRXQgZyPQF0pLvoytw74hYbWvf1ksJjbQoNUbhVif/wnCp0bX9g+C0rFlyKAbEWFBxEL2XkgyqhJO8Nd6+KJziV9KUPhgUYRzPjZgjqy+cuBe+XuZAELF4TpuOx0a3mf8jJWtJ9dPPPbRWO1WUlyjS2vdd1u0cd/qbJxOU2clqo/dJeAljl8SENqgJYUje4zxl6Al4dFJK362yCu8PkpTn+c/JQYVvMqDSbZStSgGaCmTARJqBqz3CKQ5uT/hXCdGJwTEiLq9L+4Z5O5wX3p2xPwVC+UqWC1X6xgcrwipyTFciaiObNs7Oo4a+eqEPYVGeJWL9evgZiA3meQ8G323yHyudO5XoW+n8K2Wd91sGpcVL+R3t07uMrFykonTBNnrCBrVHwua7+KjtpL6V8bA3i/1gJDi0Wikml7nCbXZ/TlATVRnEbnw6IICeUAVfyWY9ZcgI0WV3gPKcGdR0iTL6IGYAo5V8x07D4xpMSK5ZcZsLBmwq8ApivWPid35jRlDNMD+GpaiMGGfVLPA4uURGzYMNiFMUHLTjaRaGeZOAcvarVdpC9Xa6TAoFXtBVf+KfKZsrkgLfesf4+OpaiMBtyUPolPbJaA9xMabudQxb9jU7WMmVVdlnzD/b+i0SLA6wT1LKj4c1CCdTgUCSsYZlWcR4NfBIcSJtWmEEyFui4RvqFQ75qy5BTMj9A4wwFxb38IjntuIs7rEwLbOXg06TQCpU401Hqr8DcDTLHWaM4NAOSrrzkAc86xuOlO6+QqmmR9LQ5evfIi5U8m5d/4MFl+vEYbi3XCB9fU83HAqFF1Z9bQSInDB86/bmzwhw0xNJOL1PYqmLRhgg8WL02orRrLGgsSjBa3lNICu5HdB243oq/Jdh0AGF0ud2UDSuiH5n31UJb7bc6KVbtYjneFs8Vr3HmcDBqgD/q6LSdgW4yCIFdXa/G2Zz+0xIx6ogSWDScv7oyPgFD96wkVVXbhKthLL2hZIAI/K2xJIDmoQ24DNMS4kuIDDUmkDzAXwHLMxHLhdrUI0vSSy8Rpha3HigJsAMrwyHJqizC4M+3CajJhIqquf3bIO8GdfJLlurvXVLILrB2ZLQBtDEwaX2lsZi0Q3UAKXRfMHHL0+oZOClcNduguXkEY9qP0uojbRqYkSkIPm6+elAubz8n4Va6z+qYEJj1IYNeYk5+Lrt3I895Z4ZxC3NYD9Y2+gI179GPYP5L/kQbiCKJtlWar+Qz2bdrDgWmTNDaNt4OOI1cwbx9WtBqs6z/aJrnWVJNmPp5dpcwqSDkng+WCUXDJWnArtAOLrwloiC0eWkGqXLKKk5D04efxLmHZTESqqYf5aF8Iy8KE10xfQWCbDg9gkWBG49w0uogACqlGcKWXMixdNZuFIrG9G9o+0detAFeAFFKG7OHSPEmskAisnvcTBgcG8kXC//b3w+J4s/cCwfc2IqV1ZKW6X69UZjgv8bm+iqlMfGL8KztlF4IaodAepRNYABbzCxVAnAGotI5yv8G5KGMgHHTn8+4OR/lCDTXqhBpr1Qg5KocjOhe6kbeLdI/xieFUFvkvliVyur5pEE+e8XP5WvxhdhbFNqLvhBVYyGf+5p0lHU/8x7SOBX+SWArs17krO/HX2xwW2ooVx4pqWT8u6EfnJFSTqUi63zdTYlH+nwJ4hjZKZejHKcSEdUz0qn8enIBb8J+hazBKiDxkr1DNhvzuoxQv2G+zZbujqTtV7Ee31u6Wfw/ltb+TcrIK5i+rvBW/b92bx+bnCGff9SVUQGzvgFGFQoACfNWioc5waENnn52zyWP/L6/WBuUpGjkBMfzLeaSqQ6bQVNprTQqqpkX4tjGcDMSaUcgOkUbxD1D49uajzzXGGvy7MScp2DWd0Of9bXt3df83KCK5lghk3DsTet7XFKOxu09sS1wKSu7lyFLLbtsaPNVULm7hvNMPGNGZGRlbqq42RiLeSHctzOBCbLP0/qNn+E5/eo/aWiQoZAS6d6SdfHg9mxF/fIBlBnk4VuonFUdAbprPHfBV03Q5PdRARA6tYM7M3VLzsN6sM5IftGul+QfnWlZVhBiBmwMfx1X2PwN3fbBfFoW0Ju8jC1IRAIOyXz2W80LGMYmvBIhwD0sSZszz/VUk/LxSt2XAMmfU8QZCvD3lKCJDYgpbSANbYaGtwePYyguefcYXL69oA7jutiFrntMW6UiOLtlNLEnErTRLSmq2A3/Qnz3eUIVO/elsfQ27AWmAbUpOA5M/Iti/kuKFGnbi8aHxcpuStN5RNoGZ6Wpux/ADIwh+qlhXJ/Y4f7RTmDMufljwHE+jp6PkF5QdQtN9ICP3ioBvtaoAHarhhXLqAyz82z+CsIVae+yFv/up2QIVcfO3ug5W4S1TpwckeaYHuJ9rQxVcYb9fXIjiTXUcblQ/iJNd+v4TL+hls8XscX3p2vVcVJzCblK33YAqvnStwY2L5BwhefpmYeDByJ5vlAOmDP0DCLIuvxpwdykJlb1PlSE+TEbVrYYZHyA9Hs7wcNp8t5SLZ+Zj5Usb+l5F6jwxXc3yZcbGuqhHLSI/jPxu/ES1GDEJo2d0aVB/BgS+R/JYMO4Ph3kHnISC8XGil0/MRyViqwmJObpHNrWZgi496P3PaGIQurTFaf6GOmV9qfLbsIbzzAGZPSrPXPvQ7JeDFcwWyyJ3zuGm+DIuFZtbT6FJKaHohlhnxjRecRKNO/6erBYkwa6S6gJg+zMIV+tzPpXr1KxdldZLWPGIvymPvFZDgwMzSSkr3JgBCpseAiSlAB5Mni/DxET5Fmk8SgfpjmqlOppDcNfcvZOkBebWaB7yevVmLVnw10zHy7/pyps+wAZw3ohDqE0n9yHYPxUa306kt1iOQ2aleRJl+MZNbW9IC5p35jkBqBKP6ZTnjaBpxWPq3wBXB3d1S1+eUNPtcsE4uEm19u42MxgQz/jpVYbFomFZcLV5TB3y3qvFBcDEoWbW2mX8w2UjAGb8Udvbka1/hwVWnZr7sblYQCH3BW7dmFTKSh9EN2XC+r2oD2CslGnvDeRBACUydY96X7soVA1krFYZbwemawbc7SY58G9WZuisM/vSdRJkQ+fjYIjngbNXan4UWt6hY6KMSu8/QfkqBfT0C0po2t1CMHVlr0gCgjkgk72LLZQy+vHFZRKpcVoNFk/jrGhf1UIWfB5e6mvuki2vFEl3bC0BjnPCXdjze5xx8AALX2ZxiQ73/WS2Hf2jCg6SJCh3WAoTYqVOJAyPhqAfphEhRbalqY1Nnvw4rURap+K+gbBB2k5wxuVtpOTdJaJzPRHM6VaOpCLcYXRuSG4ywfmKhZ4MMkwCO93flstZizw/fMpdTZHQmxIQKfGnLYH1YRrKtwQVNfsyLpUv9ImaNc02iow7zspx+H9RGNo5N3YppxK3WFYogyaKTg6H5kvnWGeq5TDg1H28RXmi5M6LaL8gmwxqdTx46+8nefiQeAyOEgBaZ4O902Xxg/6K18mS1+iPElbzSQ+733ttY/bQQzptVaZPPnN/90HXwyvumAR5gbjVEmSU42eXwDfk7ET4TT79+f0+5q0vpo40v7+6ufFLeDUX0r59UihWGbagk0nKTjd5wLUogGSOvXUl0uRPsyXXtZafHF6xI4m4H4i6VcbcJ/nhNGF7gBhI5onzzI1hQwTUA5VgqSMDaIvpDuGoAGhivn3LP21NcJiSgF+2PDWCT7LDSaZiJDeyW6pNy0QgQujkgODADFbInN7XWhqZRA4i5sAAMDHgUy03AtmQII7WGnHIJMvwt/xcJfRMCIOlhA/9WHl1t7xqBuHQrmvUcPtA1pl+Q4JzBhTCJEJUiqBzBb/g+BCELwu9phSJ6nJf3hityt8U20WZUNM0yj99uvop2Dk37fTD5HS+saub0Pgh7s7Ie7NfRAOM3497yOS7/335CSbhgnX2enFmUX8rT+0Mxde8cUV1x/ivBlM/hgTpcmry/rF+xN9QP80xFAih+kDreH08TrhNuZLIym+wO/Y95Ej785t5IDmBmKPtJ+QspUPnDSMjcYZ0ExqRNPQXFeI2NrubNxNuKkMOoDZugDVlTc25rf2/JTzJltPEQGKOS7PR5w1Lc2GXF73o4py5cULflxnF+3+6In0J3kUZXPLLPsf/KBaL1Il2Ion4o0ATW/KjMx5MzU/WkL8BuAvpF2/ag/B/IhJDp7cz4zYZYGgCh4dL2FUDJDr+dAckPXrlcP9ZXZd1QyxZEjf1tWmeVJuVJVki3+vIMKRIdByeoJ0/MriXwp0NjakseJfzzPom5KbiDeOebnoK1n/pbwT1Yn5nJinR9LKBxGHvwvNFwkbwwqSPKN5FnAoqbN1oZmVxUeF1VB8SPgZ3gemGvxjVxrc5wNBKQPPhAlkljLnXej0vNYx9Xu/A6ZRasJOhCafzhlFrc1r4HL55ceGD91GX+YbOOTOnSGdBPfaGGNVdR4aKlCn0jrbCkp3v6vgleVKMVIS49QjC2MggVfsXjMs3Ggcx7nKi6jC7TZCEe7WM99sdR6MxAb/wIMPfUEecAvXipABbWocUm7mxs3rJzLvTIVcM3iyzy6vZo/GweWfrJ+6crqa8FuhUQwGGOdjVWdOs4qQ4IRPd/jynUAorLvPcAwfFkgGiNHs75VcrJncK2aE34b8w8Nidqoy+XWRko5llP3tfp3f/ZmI/jRvQbFPFqYfoH8X+/0pMYdjcf/I1n1r3qAO2ziNLwILVvVDnC78Lb3zLircLTUbJ+HCUo22gQ/ec93GttUZZrUZrs5RSvmBlzQmdJg2jbkhZggUAvh4u/qeWG4cpjhs72AdIyq/6dhHyEPOOxyI8uCeIrwj/ohFz0JxR148XdvUTKqfFTW1f5JDxQc1y/xj9e9mbq1SXN99OEzNkdRSxBrQVM+sf/P0W46Bhm39/hYFot8p8r7LwAAaVSmm28IkmPj5fc61fMHHLyk4tuHBQ7wdEpfcaIE7AJArD4YAO1fAzikxzvy2TTz4l9g+vemDdzdc+ejW2bBf1ie0Ga/wdxqo+Xr7xFIoSJxI7BvX4wl0t9Akp1EwkU5gQhFFAfbYkj8Q+lYe/Rug/L8esxPDng3J0NWk3j+gtMOdS4DQsKlhEWAcvi0lrQZsc6/51Nw/8AAFQ8iD+pszz9otycrB6ITI7kEV+Z9uuhRfPrToH+y0zOaFQ27MlN8Z9oimsDSqvZ13E80HYpLiWy7+GH/yN/o63yDD0hM6bwVFkAAAAXv8w73EXwSITErvEMNsTwcihIFJHUBeGHknjheB8P/3HDB5uL+4Bt/CTsshniuSS4XzHfKXQ9tMnEhPsgfuXlG//2OB8AjuPO/4STm+2xBLK4ZFeQ8GqjFsXJtsh/5SMAtJL8bndMDwW0a25y3I1Zb0UsMTACyvcPCVAk2p6NErXjiW0FkfIBXWg9GtCX9HyZR4gACRihf3O6HF7Dp7Lu54V+83CJI7TGLq5Q2Hij2YRliFFZ4EhfyU8mynIGf13O6f4QHKzGhiuk8beDTpelmZSJFfYVO3lJxSrhzos4/bjakVVu0AeeUfeLPSQJI6hSoXUdT6SYB/O2fV+AZkj1F6MBenJnhTJ5x7u/LtqMNKf3AAUZ08mzLZulE/UAATOi+gn295Fvem0BNmJxZ+UlJMlRF0U8yfmfsV/HAOIN9skNiltdv/dZde2R6/jyOUD+8PfNTVm008/kfz4heC1PvIUvh2hF068N+FdPWv5NAxMtj0kXCyIkSkMsXHn67B7NHDYrTjNYKVnVyAosIx2LNhfaqRaRO4is7+LWI7f7bp7GCDW548GPe7h2F1adwpFBKbDVn+9g1ykcL1OcSb0bFSf3BtlQpu1b9kY980pXjhbLSOeE+n3mT1n6Vm7pw1dIiSAe3K3OpPP4qoojA8aDwfDuefLcwXdzmvzJGAC3ee/6rw6Dyn4zC4FGWak3AWzgeaMbLjAJZMbj/WkYxXKL3l1PvlvUIxG9g2u1H2J4nSOtuEzRJ3CV/t7DGUT8SkafRn6QSQWFyTCtXWwAp2lTj2h2sWPAFv/HMcvW7D0YoGMyhcSYmzAACjyE1DFMQEYy4aWunF9JKuZ5VJOw4yEJoAIy3+KC+AJu6aTase9vxMwSXxuYABoCUG2KL6nTF7MudXej9YyUTCDTOMmZGdLwmXmh4Fdox5W91fMMN45ahM2tWa1YHxnzNvjHRevEcdobEO2IThnGESBm2FpwVjs5gsCZ0qiotppNANPCwvnH7Nvw/zt5s87qWjOHSqx8TGL36V890UPYF7Gfwyhta3urPILj80PxVLudF+Wus8Ol14NJCiwy+kkj1oWbwKlaJ7YPDO0LBEtmMZ2VgurJ5ZhClUUUMSh8NnZqccDOjuhWoBDLKHUw0bn4g4Ubm/9gDxBMDfQZQkb3iNMhdwAuASjWsHHSH8PBboJRld0YFJna8MeEQqoGasmfW62ZqiWKOoh5hmJKOzHxbQBZhqF0UfSI9+kF5urNFd5T8XoyQ+Ymns6PZ61jdBGQstHAftkv317mdsw+NBnINk32znirWwbSjxi0/YlC7+e7XyfJRQrWvl+yhqCYJ4DAEmroPduN5eKOj13vu+CTIfoCEZzZ7WUovQV2f7uBwT/2xVgsSZxl7Ik0yMzs7EQTO5DcUE7J0rUmGG0dp/l3hml9Qc57n5ZKQWmuXmvHwi3zEDn3kcy3TnfqVXjGXYb1dx0/8y8gL1EBS3u2SnujvBL2tRCVUl2pJnzKks5mhWUgB8Pv5KxNb2swYPo5cOWi+JAlGKvVXs7Y0laOtvVFgGDyeqXpV3/vCABRztnAbEtUbfJEDI5FGPrIDpE7I2sk0r8Ue/LMfRsP6W3B11h1cO9vZcUiTRbzfAFQc91lQuGMi4jVUfJWbQuvPYWRRAiVWrdJPGEUFTCBre7oQ6iKVpEZl2HVjYtEHMMxF/NvtRMmzfh2sea1xawqMT4+GsarRu7XI3t3PGmUJLrC0GHHG1lMHfFepMflLFcAWa5kmW3sZXf9YipfJsQAkiC8PKthBCfJFgFbC8l4+Tn1VjcbBlZcFcsbPW5uQz9la6dgrzBar78M4ECNRRq3wwSImZhTduYN2owWJlz1QwOiTAmBY57qlVd4l2ibBdnD/ItEdZrXxS2ty5xDgAAIsdPydyLFU+JS+jfbfzbRKFEmh5R2cGzpKjFgq4uH+u9J+bi6CpcWEg8iA0nJUrZ818XVT/U8yD/D3EaYalQWOOeLo8LgrPkCOHQGBX6nWkUDHozOIrsa4P4bxE5i4UW+N5GBNRBcLcZ/niZMv+KHHxKb5jYlZ1+T6NWWJIm3IqQa4kBIvDyrQyAlj30oK/YUeiLj7oCUIcrIG9Mo0NhJGD05QnUpxFwnXGqB9m5ee5M4qADyWWTzV/9OYXliwjAaHddi3+tXzzRUy3DWFp9uCKcQdbIIuH8KZQt1hkC0LZP1XbrCwDl6r/o9HLu0eLlOCvVN3rzhHq8ycQuygNkqnGEnylDj/E7TPD8OspjDf8DtymjSPfcitNgh5PK/9/sEhMepfJwQhGPdy3IIKwfsIuyB3UPMUKrV+bF0WlUJop4ohrAQNshOFBv+oZEker65En+lXqY8IpInO06fJ3qipZHb2/8A4iqTvaxBblhHOb4RrWTVsboto22iRvxq+SYWPyV8le/Gr1AKH0whJ9fcxAaGvrPfjn8m2xheRb2ygFq8TGiDvADTWsyy3iKZ+0uPgWxTLnjQxq5npuyWgMIdbIGjd67MSvmcjTasz+wRddDSt13sr0hewRpKyQ4aa1gMImsvB7eegt2DeT6mutWuJvwn3lYtE2ga+nXHfST/zl7UAouR1AuXKfslRrL0ANzLTilW4wijzBXDQrr70FogxAlVIHnP5itR05Diq0VFVpYunm7Jvve7ZKJrXnOq+I+ZU7pbxbBDOGsiUNwRUh2DmEzEY0w0RktBzEY4bB81kg5xDNajCC5Wv7/VLH1oZlYir2OeIbryhB/sAs4TIXqtdMPCksBP0JoiwMKQsJNTvmmbcE5sZZdy23Lr1zPAeaWK7D/+RHHre/CfdgQRmT0zuuFS9KvnlV8gGmpwc2dH5tJlGlH5rJ5XatbP29/9o3Y8o9TyKAW0hdxTUH+UahAwrtwE4UxNQAAmJHYta2uJnSYQGSa81xWdiMktALVsmAJY2YoTrE3tEhrR5D4QDzjmkDfHESwpKsWvrT00asGGpf0fix36eJiwNpEp0zexf6MIPhbpwS0WbaT3iWZ2gAHq+V996k9/dNAW5fB6ti2qbckH1s4tx1fw6B4wP0cKeiz2o3wX2sSOeYkFGG3L+f137YfPyq3T5nkobFhcfJuspje3uBxAOCr90PF2zkKOv0tPBpQ21FQ378PoRwbdCZnrOHDjc1lipWs7IUO/sPtVwbsst2VWUBba1mny2/agY/N4NvoMv9hh01s0D70etWSbbGm3jhcOyqVVOtxWMJYrYxlBwm0by8y59CUfAAEeEgzqc+DwDjw7mbzNRAViL23pumOp4IjcHjsnmmGg0N3cbBKPRDW/FvP/ya7AIh9+CPReLnr0qerQ2nVphmO1xuKSa3c63AaJcHOQHGTPjXlq8fV3GExWRG8eZzgs1WrIMDmYGLUs92XHyBZofU2qt0QJaKPBQJFYEUVqbGQDtgsdev9gGrZVIBMG5EbGh3oo0BK5Y4EssqhSuPlpMmnVTPe+8/75tJT7b+Z9vEvLmFvnd2KpabgGvajT2rx5QqRmEpoMbQWr+TnHjpoGAxkAELXlet2tSlfqKjwPHEPt10AYAPYX/zbaA8wkcPWcbK59HkMq1xcS+JnzYv4cRA6bTB1ZXJ9qFx7M44iE4nFheiExZfjEqJ4es1NOLftKlZFE6gAAGOE2lCiOg2xg61Kpj/5CAHi9LzSnixyEqcso+OZMRtX6Y569mjIE0uTJYF1AJCneFJSodfoj96yEyMAhLwOEojRRku1O4/bPEYa6Q2xpW/g6gh0XYmj0T2uMBhmq2LD4YJBaX5/3CMsyOkaXNHzobLqUZ2UpdlJPMLzOI7uyTiItNLznogNilgMIkAbQ6MW36b8+yfKuX/JevR1ECpWCUMU/ob0axZ21AvcSvcq7qzuTL5acm97jtMd00aeWhO/OkQcbsmfNovO+GXeAXAtnNwMOXkTtQSgY0cZvmVENI8ubCvMd9I6c5gbs6LALbQLez2cbKMa2WwMW6/1di/LD2v9otLLKDiBQrY1J64HJOLZqjht1zq/Kv/j4nEOGxeCsdgABkI//pQkUMiAzfW89Rko5BfWcO4NuxR4nphJW4jKFUV7msKoXuva4YFuAH1TZB3SNLPpO1MFwixipFAfFQi+HRAwLsZEKK2tYO0iX9h4LaDyWEN8jHzrct06hpYBZpR67ovy+pezv2M0qTsp8s6lWVe6dyaFKCqwtYAbFKlYeB3bPBxiANMZ7aqoKiXhSwN19SxwYoewdWh+HPTBfOJ68owa/l2NK8mP3q6wjHQW0x3u/eV3EKIAp9iBkfo0mEpqqLrYFvrHXDCwBAFzcb8zsUAj0CclbDxL8yfBUMug5//0h/f4RlKTLcEiCYcna1bntyW7DpCQhducDsLe4lRs7c2xQGYdUjgB2YYmx6gCYy5BdlCoLMI5Hq+/LQq7Ve3skmHwM/oeEkFnNKXOtE55Od4L6Gjhn6vcIZ/qcFdFNrtWPjR08P7FDwXzT0azVxBNywEcWP1gQy5GfqLWPeNg2lJaWU2iKjlEXYW+tVEAJTMVTgrYJHriuIhtAiuJLNF02mLQ2uPaD2YTPEPcIvkpvIbwKh9u3x2g5dw6ohGS9m+vYF0bKhJNDMVSc2CWxSGlnKlVie5JIgPCsaOPbN8xgVlyKo3W2EbRb6mveKOGIPpT47yk1iKMALofD2Kwo11MrtkJzadCQ8GI1pPGoDEEAh0Wn/zvoeYFITks7yzV5dJjRncR4SCxpTBoKnwzmK/X66PvlW3E6kVdyommaRr1XKPYPnDGj3J9LehVOBWw07sXAq5FxFlGHH1q8PoD7Ky8fRyeEERhRgijCrlMl7K9bxIzv1qWzegt6TFU0BdFiPyysPpHVN5Pjr5ZG0JtHAxrTFZE27kUb5pkfyUpNpS5O7zC4kYwc8XgGKq31m/mYGB3/FAt5GrjM4C017Ib0Ln+VkZ+Hn/3CmvPZivZ/sY7EL3cZA7lv4qAofiFKb77scoI58NgAk/eO82xbWzVXMBKnuK1qYXw3t3VvAfVxuqQHzK+J1IIQmes78ACPkk16afwX3qGydpv88iw3/cg05XhtfHsH5pIHR5ILW4Oq6cHJjzwGYs1Xaz+hDoW+XRyh+nyYMOU4gBaafAoDkBPEh3z6l2usBKR8/YHyovJ3KlpaUopI+Mk01MLgZhEqXLezRjjEnPA1NJRiJgO4E+EhwLrcSetjuCV0p2ChXd8Bx0xsbjfn9fDyGGfHFZh2slkJQHpyUXU96kO/bZMx+YuW83NTOC+CGkqM902fshJmY+LJfTlbEKML6n/DRTTHV98dKb0gk1OAF57WwqOsBKlVZjgmfIwI2TBJWYb5NuNiZBKA7+G2U/96pZ/gCDV4i5vWcdPxvGBAVgth6ilz1+an6O2NvPyHlheyq5Zta6/2OJiWRKva72aqiDWMtGumtK4P5bqNtHJgMB+4XDrDF6AjGdZd7jhHlE2A0Pw7dZfeoK/18/R+oVw3RknFfOheLTKgXnhmgZ7SElBUhNGv+dV+uzdu3+iNPVv1xR41dIx4hbfOgANgx38SyLcgO4ySXqBUICtFrHYZi1UfH8eXbGjNce5NYZznJhvDGxRcsMm6u/1L9uIoAiPhrAKU6e5XMgZJVppepjoGvFo7pgQNW1k/BtpkWZMmd4QpvwsV/arZ5QlYdtUVWXVmC/9meIzaaKs5o/w2a3a8TSoFq+9BzpdZVYtmzJuufTR2WpuTIkeFhc97BdOMIHcETNzs/49lctCBxdI4K+kcdYJ/BMbFViuzeaOTWfElghEQqulAeHCSmjynJEqhO2T5dP9nompLMhMSd5ApLur5/YGV96jE8OYyd2dbyeLPF5NeWviaE/mzD/6YUsiovFU2udzUvE8xpq8CXfni9LMlM2s0xlcTuGAvw2pq7VlcXb6co98Y4SGAQ711tPI5A39k50k1W5xKeZKCAzuRS0LdQiJca3hcDVKIGKbtyYApGpUSn84Yy40IxGM22VHw7XHI5X+/y1CC+e5Om+3yo8yFcbZHaPF/FDQzp41cwqLx2qRzk/a5LlcwpYNyvC7DiW/SP52N2kDUNWqn0e/ZV21xcFSV50KIAAj+2xz9r4SFMqlNpQOmgy77GwPOGNlw7IobaTbU+Zfvyb2pJa5B3fcltQLc2js0M6MfK/toHCJa7TqJ3VygXg6Fegn2ok6CULk8fqWTsfbEkcztlGeEmLR6ouMnyOga+TRl9C6e5jLGUGgy4oHvlfWEh0QYiKAd23SNXJFFc9/ODlYYCoHK9DWz5+eaniege5ZU1UJ/5baC6svSc6F3FYxEBZ29HX9PLf2jx6dmsEk4KtVJV622ZDLECD6Q9pvaslTtQjfgEq2+iqwOiDYe8Fwy3T3+63pTUi1ppiigjnf+/O1e1X5fOu2YNp+t0xqqL8dDxGjOe9AHquqm4Khtn/ILLQly+TzxN1ONBhQP2QUwRyn6+Oj42Ed35wiq1MAsMtP3rwqXXt6nEzJREKFhaSsA8fqylaeTjYM80NXaAQGhyCY6V1VsY/uAba1pRXXscU7t5e2H+htvsiD2QkFVu55fmPP4ycnc0Df42+7vez72THk0h/c+W0k4nVvqyfqInu9fp6ri9qL0Pdy0vyIay1c8Dk63/rGz5d0tZiKBCQUHnKRTlzT0eVbPgLqc5a79bOF+IADZtZ7FwPeiWbcfm3KqAt8fhd71Zb+5XJM1v2OXphmDrBwb1ceUBuba9caWuSEm+enjHoq1OfSVr3j6KlLzEm8i6oRkUgoMEt4P+RSapOV/0RHon4niEfKmwJ9W/eSxesq6PEXWy77+U4pg/srxI1isuIuz1CQwpxQXIK15ZBEyGfQN+hBcGcanLVSkNOzOE3255/DGbNpNn3uBdk65wQwqjNQPvtEyQ2IWt+uTJma0asf0F2L3gjZN1M/z+PfYuDRLJbFO9oWxrbUePYxQYBMPACwBY6sZ3QbpW/qKVjBbMK+6VIaSSxAGzbzXFqcbnZ5ahcujDtV0Zj24Cph42MMirL4zK6IgUev8IZWrN/qo43ZVqy0mhnH+e6uUFxjbM25TYY45NX2BTf6cWJt0bC+xF+vXfwLXcuVO4KBcOzMO09fucCnQkMDGB7ULmfnlOQH9HoiRPzkQmcZdimmYb3KfQQ8kkzEyo5mGJs/lp3Qx0CZBFzo8G8MZvIQzeMRZE3Y2Uu3Rkq83ppZYMV0p8soLavvfVuS7pwmgbT/ghSzm9MRO4B8AHEHSwGydAQVA4MQZ8zpo3PJ7RcPXb753NYjIE98OTa+aw2iMOQ3dkAtNwkHMngEQJqt4+QP9dMzNZ3cFFVBzWoUu1+DUhH4QuqiN+7L/MTiemYyQUB+KACHrwV5lNgT8RCwS8ZRadNGlYvlfSfemyUF5w9FJhrTf+5VYLRV2jVl0GxNtKuHHemXxt7Mf3WQNgjSwc8lKXdiBEn+7gqAzpL7cTSKN4hQDwqy5E4lOoIJ7acTn+GF0ke65XGXC5/kfkDZBgxQ2jJkJK89hPiZsHMW24ayOhD27Rr7/cHodAgKnYSkBRWAHjaDghL50DdEexfxZwufeB8+t3pio+Si+m7Bf3xWEuQqnTLX2a284p81Z6SbdCcrRqiMxYyof4DXAyEOgQNad0GJ+ZKRHgMFV6d9dkljOK4dvh+P0ZLTXT2Y+CAIJlLJITwbiJdPs2Dez12nKjNG4teccxcG1ljC1TxRWW5cVU68kVEC19EbFWEpsc7Vd1+sQ2gYRMG6xJ90bf9Avo5T7SiOBROQ+pZxt1y8IvQhwsrEqMdVu1KfwK3ZomIMHciszQbur2nM/JYVgMGx91MdYY2N+U+uAh6X7zjkHyT2wwm3g4hGFOAMjSB6uPAqCNQ9ZKsrDjkXcx+bV6evAyVVLObFOR/nCfb7fZ3Y6SyQnjS9eeHeMfHCGbRkbm5+tzvw0MscAMKyq97gqOXPS5i+Gs1bq52m7Y2vDSh8UijutIh0KEm/IjV+wX79ktGVjUy3hjEKJyFxq+KlFwTUNC4v7PUxI1PDmMiMXh22CMyDj1aT1gSHWuLN+dpLBHXaZUb745sF4Py76RZVv2rYth3CRCbmM2yZ7hS5x5dqSN2Qa7D7bT23Fhau7ZBGUw9ErAZcRqYPohBrK2/vSHDHHbCnSmNehXz8h7lZTg/l+X5NIbq5TX2nH7+04Ec830WyDC2rxYfy08ZFc+HxoA0+wirF4jC9wI/ZauzvyXIuzyoBZ31cxwh/9/hlvkYKVyKVCpWcs9JweyLVPYHISSl7wLhhpIchony1x18+p+oVA5LPkmxqDe/TgCTqtjMcDb9eHLNsPtNwE5bpDHzMApUKJqzC0WU3av+rGZTSaJKm6i+xw/7/aeB2v81sKp7H3SpNOYB6R8BQLEt0qVodjtnqsQQgcPsL+ATM6yCm8GCo30x3nUWcKLR8pgU55Ni31dF4jx19r/4G+vOHkyX1o63vWlmSuR+0uxuTP4Ii4smZYgFDRO1qIkXUGxO6Bv+OJ9wxf0+WDuv4ntJVPoOMF6L1gJ6oA+YGGgdKM26m3BaWkmlCg2OLTowCHnN57DYrd1Am4GXsfpsVRsNYR/MnaaCZm8EhBWRCd16Rr9jVqvQHJn9R6JrFfI8JaiQ2lO+R/qNyP6CkThG3G8OUVNJZGp06mGs39WkXxlcTNOKKzLHOVMW/YGMQCUQhll0ece1SU6+25YlREGu5g0Tb2h2AANhC2EBEWdG0h1gW/TCj2uBtYHchI5eEARR95/5InGJkX1uE1id7GhQrugc2YvI2SOuOunmI37snsKf9x37EkDkb/DI0W39uOZYcpxImMPSVpr9BhD/vv1nJjOcEHN1D4YKFWcddStDow2J729wFlCUV+g/c6ANxvmA3dhFROVfAG90aQ6vwrBHfS5U/DNV6rVjFYg7uQzNfeyguPlpbH18F+ffOjHI4G4WsmOj0aXapVWqXADR0wHBLxfzkQtP/5AL6g7sTF57w2Q5V22c9JG2uxrEmxcNU7ijtQ6yQjxu4w86z+QG2ldEyoowFeCdkDevyAwaHFm7A7c5d4BH9T8xldR5s9F1KxlKbUdNs6dZv2Q2bpK3GAY4qV3cp/VSJD4dl2KUrkuArENmIcPtVFuFv75UBlmAQMSZX/1F+834C9atKTakRG5jaZ2HtW4JF8912x445JfEl3Foeqw7kLurA7hzbdkY91iQWJqpYhJhdxutkmRdsO3s6p9QPiADHHVPGN1AiyRVl7RxaGXcb6UE+3nB6/daUj96WRm5wf4iAqTSKzhTcGhEnPywPZzZPPAFZKY8DUFXZY2UbBE9jN6zLR2dpoP2e0r6c2vJqy54glNL3KZ2t8fyYG/jaiOghclfpd/fJ05SVwx9IT7BR7quU12BmpLZrbAmKiovkQOpo6x8ADB4KDur0VR3mWc7NJVAqv4itIA5XeD/Ne669d8NxicEtyLR0MoGbOMTSUZaqVUk7ajKgtbhrVAum0iVsEYklEf/sk9YE6YxXQHsfRIupufdy0+IEGelrUj0KbSMOB9xgCRzctqOpoGCp/baG7tZbwp6mRPFMcH/wwB3g5mKMQInpDVhHCf9CU2wGXjagljE3kGPyijzYuJUASvjEBUFbgAD7gYbSNRckAcH2xlyLzkskzjEEj/RK0QJbHeMBgnBy4rGf1F3M8UGzS6IYu1wjSJHweauqsVC/XB40q0VoDkej1KC2Qg3nqvjHSSksHkao2shAzKgerSSV8bu8Zzic6TYZ/LiZgBM6kw9iJUcR/4xNmAoBI4azrwvgjZQgBlH1bqveHLAF7bcF5SmAMv7q50GYkYlVIMF3SIsPP99tl9RUeSb1I83/DLuX4rfPyW8HHvda/hShiMEF//8med9s590/EIa4srb+9f+fZKN+Xpner7kJZzgPAFMhZSE5ud2qV44CB0VWGOP6+e8fZ+K4t0BIvazWYSLippT1Bl8vTth9agBzoUlYzq7bn1fas4fMx86txEiIdFfWNMrGvmu3hM3e3RB+70l4I/tts1rImmlfDebPHtWNoJycoYm1CNCVjfXSEBbxAHgIF9dtDpmOlTH2/gGiT/sxlI0wuak2Lw3d23ZGzz7eq38LPbo7ahT12gmVVX3E+R4zbwjJF93Bb3jJ2v0v5+3kkvi7p5FrsgfYt1axF/c4ulnDqoO872gL5ZAu6po2NU1SAcYOnBXJm+Qhe3SfRp2iLSEpc+/OX9E522HVuFgpR/9314t52eGoDmjlOp4/wr8nkL4Z0SPZ6AQebCAEphaTrLfCEApF6gzIch05rouIYvRrnU05wQsejpFO23rict9c7wLRrbGd36/MtmGIlN1wR4r0LTP9kJqRKyA+hVrThXUwfuL9yq/rb6dnJvdXMeY5g3EegBkP/qBNmB8RpCZW9Caw3r32hgBd2nGdyyeU3hKfe3DPSWiESXa2XmkQhsfFTBpowbmNk2Cfw4KVy9j9xODv/HKQAFamp+bzLSd+cOYRonThVleuHqZJ7qH+qvp92TBAZh09ygrEVI+wlh07ANeHik7GKqA2aU4M2+6h0/qxUCuZQpVw9qrmX1ABLbNPqNCltr5RxVBygGNpIffvlm0B+a15VlCfTT8EQkvDhIfGkmlEFJ5jh8vDweG6T/LeZ9fN8I+Wk5+JsJo0DZBdd4RhRn8s4ARP1YlIZZjdhvR8Aw/4EHpVXIpizLVGFT1shpS6UNbSCtagmjpyT2/rIpAd2ZHy9jSeELy0nr+DtHPqr9/ToFcULrifBUCPZAvK+dcQ0n0Knxk3rhMurZxkNGXZCeoEj2V501eqPbG34r8gN1PTaqWWvHR/QmkCP2gfXqn9Uxi2rIBGuBfhgekXS0SUCJ9I32KQX9TOVUgtZX9vdewzF61FzlvqTV3dPtQ0LjwmAQ+lIv76BoDfP2+QDU5YgCZ2fYtQWCgsrjy84N7E2KsZrBWDXegmgZaJtokV0yzX4jKtFl0fyB0GsFqZ4/iQopC/LeHOlvGK9E7VMj9+VKcoCD7XKJYtrIFadvTcxjZ0NzWDLXEb17DH6RzGkeTQjTElP2hFTCTBO8qfBvycYdEkHhK0nm0nKW8Zi3zvI62QpTeCClgJ9v8kUMgyaLEeCVdkEv6pCJ7D2lJ9IOwJA5weuLOtKhFuW/YhSgDZp0XjqY8aezj5bxr96HQiFgYIgEg7jsL5gtKumX5lWKqBoeCJxH9r3ofqLRrRCuKM4zLMNzUH/WIZJl7XAeJMELDreTjuZ5aKwQPaIexlC7jfpd+mvGGwzC9Hpr+96PincchH9KZm8fIRS3CmC1W6e6vqK2tJRuMJG5rtayohYsk+QZuEiqPBevfp5N13yw8zirI4K/pGrJYtkBmO/SwFJEEhHc/mQXu3D/5EGNCE5+kygDZLpJFE1QK40pktWG9NXs4kgFyshRc8KYsPT5pVncM4/jlFChmBET/OpckBWoS46noBstnUDZP7tkVMR7f0nASM5VaBzd1vrIuqEGSusqWxuWnS4ZcYpVVD0jFSy2I4CyOsiwOIlZPEpwjbPhOsOCXWOBuL5hyLIVDJUAc9w0kL8e7rGLAdVTtOBV1f67DFEBG5KB9qc+mxMKtts0UOSqWaRIyz6uDQR1Sfx2a7damFBOCsN8YIaj7sX9I1GXypkOwfbef1uJb3BvV+2aR5Aa0wAUD9v63nAOx8HnJ1s10Hj0zl6+nNN1rnJOhFPx99Ingi+yn7FJ16RSmgYpDs9LrCf5mH1EvWQJcSqQR3swWQ5QTYK6UJEeolPn/g0AV+dbgvV0v3YMe4jSSFI8NimghiD2WNBIfJLwwEDY+iDtiowaOxkI+tSoG4gAu1ME8Jv/ZWcI3ythVonMTblbvjV6LwoAlRuWmPwgbahP3jGPzvdhQVrgoUDWe93AxoqY1ZLxkJI+p1z+IZWnSV09Akl9QRyBBOC2c9NlkMOWi+ZUqyj1RGtogBEnI04nS4PMmVN3r5+ZY042pVP9EzZ/7cZ5s8ca0bjSnt0Uff7uSZk3EBhmpzJPf4wqHGoVQ79NL1v5b+zN+AWZd8Ljbv+7Or9BieAJh5+IGavVDMv/yktaTetdVuyWK7uAYobkDdOe5VdNIaxx1L5AEXyyQ14Q1vEUAFxTn0Yq3NPmVYKxkkjs1UaAKTrgkNVA3rymHdsgiSDL6xiBWjRcxor03b7vfVHD64VxvkkVbexX3JmIoSwDCvGz8RcgHlFTob26uDLPpOg0ePw9b9hbfdTTABnhDmszdl1jORpCIvN/YK7TpLrgQvdQe+dOOLXIrIlmff0oFeP9TWqS23MOQVnpl59KHN/EuagXnNRDkhzy5dzaGEYWndWh/4q1NIogSkgGltW8jYfkPSM1rpXnfx6r6aslLJT2C3qDGWZzosaCCxdtMXy6fgxMF7Qf3O+3AplBnEQh/40X3nLsKJ8ghvW8QeaEoQbjSyD14wUoMex2BWelLXlouFdZZkMh+PoUR74vQwFNbHZF7QVu26TfKxQhDZ3KBH1vFkCei8GpNjy7qtrgNmw+UTggleIAAAAAaIaSP1dNpQx/NsofbKJk87B5f3/55xi79ypDXw7W6g/U/uLMAmSZXWLGuv1SBqVYaiOVM+vN8Il6Gdye/9YeViCHYhdwD3kRpYXJq5kFdOf515HgR2WqM/uOjtck8vqM2RdyYKlP9fgQa5eohfqQ8kE2jrFjpwaHItQq5vfSzbl514yGfRPIcR9ozR7mX/7kG6uxb035yFr+0AARQRTCoAAAAV0dI40cSDraXOLbBXA7CuB2FcDsK4HYVwOwrgdijYURe2fxTCnjnflEAAUD6kDF4jTukDnB8LvbQ2VBZP1dO2URTzUFKSUgpQUcExXrAezVEtN1M/1d5WajXR38kI5Hp58YewUhrOTKDXIZIfCIrFx8MWu/jOZugI3eAHllUIjk9835rWtBA1tS4Ql+oDgyzIVYaJJaesr+VpcKs7NZ/f5bLPjrLxLi4LHHElP8MVlLtnBcTqUkesJTVev7TPoDYSuunuM/h6pPge/G5TwMWSKBeJ60uuS4LiJbhqshoT+vZvDi00E9AyIEtBnlf/tot1N6obN2VU0+dOBJIl7NkhFpseiwVbuMZl+LjVgULoRNK9rIA7SpfWpZb9bYMznrGkBnxyXxFki5LPq4EKg1JveYo1BX4J4vZIsvxnFJ1HpwQvXEI7qIz2l3N8y9d+V1poMQJ443ifLfoENvMjLcUaLq2mt1x59wPYSmI9G/AD2zSuJulyfIWTw5ssWPvc2A1F7zfAXBDSjp+MM8BdeYYA+V2W/msSMWLokRIykNtELRfUHMWcbAL/pbZzoRLQQsHzTSdQt6jnzqC8c1pmqEp5NryrVIQ4t5N1df4gccd797Jbt7eKO97pytkqSJX05K2HUWtP3WSRDcI30lJ31f3zacxcL42ih+4i8x0wQU6ywjv0DFOZcL93Ccyj261S2+ym2Gtj+ClwNxpwwD1siwmQJzxc8U8U12uDL+wbc4Yue6wTVTkEfQ4XezF1BZsX8webAxKc8Uj5xScgBGl9uPkW+Idcvd3XrzV+//iRW6F6Mu4X8N//hNLZ8QCZeZKIPupAYIQWBfRKmefrDirYNtuNRI5cmDqly+PYL2Na2fHV2RXlidTT0L1Obi+r3EoZrnCBIgZnvK+NXNiRftPIiFC23xJD7W+wAcvEzy8+eC6MqCa2b5PpGiXZGIYIqlVZ2t3PyEMX0PTyLdXo4sqw50rlrv294piEYXchZ+ORFsH4nyYNOb5s4F3CcwIc3qNmv00tOQsDEvJJwBg9XFF41kdPc8dcx6xyUgO22E2/6S3s2Ra1h0eN2ge/vNSPQjEBHWmy2R1rSz8lQiW/5YobxTBhTTmSwKMUTXjwz7cVM5SdswWkhzFpYulznTkUWHAxSg0WPm/J8FjbrD9qRV5KNtXeHFA+ckNEOkszi/yIb4RTuvPEoI9ae4xdHf8Dw0U3E0sYQ+24i5PEHMeJRTdL1wUZ+k3ghxyKdvtwUHZRXruZaaLTmK32OdCrsptqcYljSpeIoD0PrbA2glIxKSzq/F9ZrV4ssh/8foz1Z7a18zWFP9thiFrarF/BY44n0a4TZJHK4hEUgX7if2/W9bCSySAWN5I6qPumYzGpPs7DUbEugArGGwOpMVREAPKMaDGjmn0foIosIpfzPWzg/d+ORe7s1WFuhdf/qXp+Pb9pQYvYGig8JtaRCH1Ef3BQU6VEbb0FQw9zpKTzpGOVkFPR7FQT/KxmGqzireNUt28PMYawAZNEDUwGVJow848V1VIbeest0OUbyew3rlQ+BTD9rgwTzXUz+QMfNaXfXuK9KRzo2uSggkH/TZj0PZbpkdltOu4GYfCMt/9wpQdkvMrrcbXjfqhOBMl9KcvazYKLqu1L65PPNaofETeq4SmX9QKBJOiiinr9HdAhtb45mjZMNEv2kdDSP6IlyzyhajMcdR0tzkfZnAPSJncAV3sLrgVpZN9Nd5ccT66kqDncctivHpfs4/gsRU2/va3YuStuT+uI3t+6oMBKWbrTH7MeIhcJUXpIvZK1QB1CGM4nZD+9QEvrAMSKMyeoIUl16vvEnWDZIC220AI7RJkWYuXzlG4UWezGvSV57IMqgIH5QZYYHCL3y2lxO1NVnAEb6IxTmUE3wQRuE30iQA9O/dXO9a4w1DlcEEwRfvAbwW9rx9Au198yUhJHcxkLSL2LyIa2KlOXP/6YzoMQYsr87FbkEDx7M9oc894IVs6OqFJAtbU0D2+dxv2883L2zzw+yotpBv6x6at7ZylCSt92OW4ERg0uqzah8QLem9sySj0ejq/C56qntXNEJtcADNaCUDE6TOB3v11T4/PcLk82kGqEW5LjjA5ZtwtqdifL8PZ0Y+Ccb8dUTvpLSSPY2LRYD2apotWbgRJKcgIyNtOWhxaJW0Lbf6/gcJy668mEW0rpTkoyWQSjI5pj4rH2OrybkCHL9l0WSR364MtFk95x1kK0pYTJ2y0I0O9TzphzwDbiGZSlQ5UUzr+WHV2u3kB6p4zzkR3lnCRy+xaxHNq3uxWroS+/EtTyPpEFv6/xBg11ZCOGDDRncyHT1YC99WKaszY385h7fmLxB5CFESi7s13ZmW/bGxccRF/CN0uSIvGIln4BGRUQ7WsciYaOIuQKaC8CwqNF8FC1C3aDP5uIYz+L7+PuADgT59J5c7ZyzWMDP5OizBCXfWKVkYjf0rxlmanpx68DKzem9TxvERcqcp8ZXuaXnAVV5iH611jTV1+UwNwbygdtXc4l0dTWzeUhb4BUQtch5+TYhBmvCmQxypyszOL3UQbDvcolHVEML/UDeK0M/EJv8+8+NS/V0ot92k5vsYOyrVscttcBc6kGIyiqHAvJHUoemscAW/Ly4+D4TanCvLBaHcfYekLVTcKhGZ6DddeIn22RmEFlsHDea4gVmCoACE8f4pJG79Oz9mAygAAAAVMROSbhZQrNySjYAAAAA</v>
+      </c>
+      <c r="D2">
+        <v>1775191934086</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>banner-men-1775191940125-0</v>
+      </c>
+      <c r="B3" t="str">
+        <v>men</v>
+      </c>
+      <c r="C3" t="str">
+        <v>data:image/webp;base64,UklGRgJCAABXRUJQVlA4WAoAAAAgAAAA+AIAuwIASUNDUMgBAAAAAAHIAAAAAAQwAABtbnRyUkdCIFhZWiAH4AABAAEAAAAAAABhY3NwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAQAA9tYAAQAAAADTLQAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAlkZXNjAAAA8AAAACRyWFlaAAABFAAAABRnWFlaAAABKAAAABRiWFlaAAABPAAAABR3dHB0AAABUAAAABRyVFJDAAABZAAAAChnVFJDAAABZAAAAChiVFJDAAABZAAAAChjcHJ0AAABjAAAADxtbHVjAAAAAAAAAAEAAAAMZW5VUwAAAAgAAAAcAHMAUgBHAEJYWVogAAAAAAAAb6IAADj1AAADkFhZWiAAAAAAAABimQAAt4UAABjaWFlaIAAAAAAAACSgAAAPhAAAts9YWVogAAAAAAAA9tYAAQAAAADTLXBhcmEAAAAAAAQAAAACZmYAAPKnAAANWQAAE9AAAApbAAAAAAAAAABtbHVjAAAAAAAAAAEAAAAMZW5VUwAAACAAAAAcAEcAbwBvAGcAbABlACAASQBuAGMALgAgADIAMAAxADZWUDggFEAAAJBwAZ0BKvkCvAI+VSqRRyOiJCEh8qlogAqJZ27poBoUrMth5RH0yB+6yHg/7nz/uUfAj4l9w84vmf2J5cvQP/a9XX+T/4Ps8/RX/Q9wf9cf9j/V/XH/W73g/tx6g/6f/ff18917/mf8n/Y+7H+k+oB/Lf9J6x//O9jj+zf7v/0e4J+s/pmfuJ8G/9x/4/7ifAr+zP/29gD/9eoB/6+tn7J/5btx/wn5Qee/499F/jvy+/u/uH5t/Qf63/lehv8g+3/6D+yf5T/uf3z5n/yH/O8gfk7/a+oX+RfzH/MfcN6pe6em99Q72k+q/7D/EfvP/l/SU/tP7V6yfpP94/2H3B/YJ/K/6T/s/7x+9fw7/p/995Gf3X/fftF8Av8x/uv/N/xn+k/b36Y/67/z/6j/Z/u57m/0H/O/+D/S/AT/Nf7R/0P8X2vP3h9nb9wRTu0iRdsUcXcCTW32Dcd/zVQgQ4Tbfw+qOLuBKjhv4aqKIS8EcXcCVG9Qe1e1m3+LAKBdU1VPNGDj6750Cy3bgJt47g9+4be7PViWkrFlfuaRr1o6feNuQkkEZnJ1HBgRf48rChVKytqzmXOX8g4Y4zVZr0R1zFvNl/QMDD57sA2vwvy61Ay9fGM0F2nIgylHkJMvvgWXW3QBt+DM6PsTI08794vOOYWnlf8Kn18KelNOj9pTQ56bUjAjoVGbzpBI0kI37wLKFk2P/B7MdiAg8BeSkt9dGlcpwZNXJNPgRL1pUlne8wQj7iv9Ch2Y4bZ4NpmoS9GOdxmDiz2kSo4V/UFeqv2Mbvn2D07APqHj7TtNbbQMHJzt74PEJtg9OvP7I2lLBKjdDNWhqAjJ/w2nLKZlq2OCQHgIECBAgBXwZayuctZKsPZG38Pqji7gSnvuEu33m1FVLldBGxtt3z58+fPnhO99ETAXzZs2NGSJ5OQt9AukFb67cojbrfRYw2EKFsQ1fK1J3Qox1v50eue1U7fI3pckT6htng2zwbZ4IXJyzJmAQjK1cypvuMdu34XzUiHcrP1RkR/z9KfVC9WE+r1CuGC6ZoqyLlSQcFVlXIiLxXCIiylYRg45qy5HUwhCDLbgF3y0yJQ4Ns8G2eDbPBtnhkOhqccP1FqJ1su/yH4pJ3Gx+67njS4rjaQmyikvAva4CrCh/bjwEjifyZBGv9pc3QTTVbd6eD09Xxxca11RkSMuDfpuw2D3pbmPJhhbeyhBtjGfHg4hZxpM4IoO002OAhqSmHcjMWMMCdGBOjAnRgTowKbKIJ/zGiXqo0SY5cNUk118MJ37Qi2vdQtkgbf5mjdzMLugfzs+XJrp2n8b36iJ56KNnCbm0hwzcNDUk5GOhvo9foNBjAxQRXofwmDi7owJ0YE6MCdGBOjBH21LLmoCUmGDwE4630V2TmwKx9iCAaWe977upUsPLEjuTAv9iw1zxJiJt+7cjnOUgTN9Ot7LpoOQds/0zjqFEqELozaG/3LsZ4IgTowJ0YE6MCdGBTqiHvOsR8T2FxdhStxlN950C3Emzf1abqyfbAYfYaJBPPE/MUmAFvRnzwnFyips7xM+Wy+UdpUnFPvsnwQFmfRL+rvlPh6J/63Q9LGyuOGnlosbrWN1rG61jdax1at00+xS9esi9ySG6I4PWgRZE3X0WdIolIZ379+/fv9tTrL5uvDUrfYVvsK32Fb7Ct+9TF0ek0uPSxS9q7CI9FfPYMuWNWGtPHEAw5wf6cBY0YCuNhCaUUEQJ0YE6MCdGBOjAndOVxu2qk8rXVzxP197dryXJyd0BRdECc5NgUt+8hU4nr4iEp9dCxutY3WsbrWN1rG6+4BrMbgQSG+UKfczCT9ywR/o5TQ1ZhM5A4knLH6o3iFOTtp06cNGBOjAnRgTowKdXYR0m9F3tZY8AwlIifc0S1jnVjUW83OiEiadVs6jNi88f7EOm0MSePg2zwbZ4Ns8G2eDbPUT7eeoaM8G4JTqYd6DwoSftpKhFDgcr3hGhQw8iFFfCn/ejD1U2GBOjAnRgTowJ0YJVmtgz4Cq9fGoszHcFG4s+UU/8CP4nLSRBVPRXWBFBkVoXGp2ZaKOhgTowJ0YE6MCdGBO6c0x9QlexaQ+JEA+pduj2tqjHCgq5jPkhWWCC1Cyhrtp6Exxq6RFoUU8sbrWN1rG61jdaxuvtdSgKW7FXhEuy/ahuE5vhTUqQ4Vl2dqZbNbG06HNgzxFua024nxNoSKvcj6VvLJw0YE6MCdGBOjAnSV0AA1soCVOUikkIxyl9iBRVKwMmY27S5lNyid7DvbxGOLMeP+REGmg3lZ2XpRj/n6dOGjAnRgTowJ0YFOr9/MNTQK89SDLkjbN6fCw93/0sOtpjkseHSksG6S3U2psF9gzGXieZbbELCqh+1qcuycQvUFb7Ct9hW+wrfYVvtCCBSXM0yDrIvzwRsK6pY8SlhMIPSQ5ZuYy7yVm+UHsszGK4oWAtq9QwYkvalDg2zwbZ4Ns8G2eDoMtCmPhZj5yhOT9KPkBaG4f9WSP5lRLW9/ToKtnl2je54LfjZFjb5+qNAzLoBBkGeDbPBtng2zwbZ4NwlxmeKUNocs/pR3+g4Hicb0pv8ovCxsLzr4oAvFcCdQXiHcT2BtieTkDbZ9T+1dhowJ0YE6MCdGBOjBKsLPw0uFGwcAySspcb2+3+ZTt7LdM+CJPzjVBavd11vaquNSZOjAnRgTowJ0YE6MErCXUE9C1x4dBGHykNtamaojxRNIrKZjZMna6UBuCbvsK32Fb7Ct9hW+wrknpTY7QVjbqQpMl858XDH8gP2Dlxd0YQe+QJ0YE6MCdGBOjAnSVvngQ70CQSup07mSY/ReO7NJPpkmd11VKBpfGnk/Q7AtQVvsK32Fb7Ct9hW+0InZL5P9f1HAzkVdI2kBoR62nzIACjlxCyXgKY3BXLuiY2eDbPBtng2zwbZ4OglQxU+gDnSXdoIdhV7xD6jyMz86I2Jv7RYIJ7wCAly76Zs5G+QJ0YE6MCdGBOjAnSV1jvDig7F9z7upvx4poRAU2TniB5TAa2vNV9Uv1Sp4xLg2zwbZ4Ns8G2eDbTDZbVKUSLEEY4blme/v4GMm1nPTZ99GfmDmstVTVSDU+sRpBng2zwbZ4Ns8G2eDcJjPdEheM7qrb/ALPiPxpNyDNwBmuYiIccPwhbsmaYwpTCtgiLG61jdaxutY3Ws0IuzS7/CDCGQp992XFq1EoQW6mytql/2TXxVsJuXdkrJhp3rbrPTs1dpsSbDAnRgTowJ0YE6SXPlerP1DJKNkBkiZ7rD2TQgyh/kQOSXXpmfJxAW+etYahKJ4BKHKX8ce5KGaaMSbDAnRgTowJ0YE6Mf9I//8YfPG4RVQXI1qZh/RDFONzUDWgIG/HKac1SuKY2SfNDB0l+cqryM8DpBbWW7MJCADZmKY/E+Sw3ixZ2vuvXbz4dnFTYYE6MCdGBOjAnRgqsp0Ymj/7YatpCJ3LdiShGwBA6DNKYdnCmvgEZQruluo/uVuIUfR+MAbBCMLrIAGosxn1wfnwhGDbPBtng2zwbZ4Ns8MUHoXxvXr168UIVU7U8ZUWVqzxoMYGOpJqFGOsTPgZ9Lh0RBPTpw0YE6MCdGBOjBKlMTiqvorM3ZSpiirETv38yk0IdODdqfXfCW4BpN2eaeScGhJLvg6kDhKOw6B24XeoBjBGb0iyBkggXhjkDUFBLlI11rG61jdaxutY3WsdcU8azUcJnVcecn/hjIZej+JYkM3CLp+gkrVfbS6I6Va2m/DQgwoFKqGpFA3jZ1vmSjgDRgTowJ0YE6MCdF7F518F43p7qKcxbH98UHDLd9gto60RKi30Na0hChbENWXi1x4uA++bSVjdaxutY3WsbrWN1k2wQwTYp5qKpuyJUcGk6cNGBOjAnRgTowJ0YE6MCdGBOjAnRgTowJ0YE6MCdGBOjAnRgTowJ0YE6MCdGBOjAnRgTlQAAP7+2+z6zWZrnnVESkgE5BT7XoZzrisUGwYB3IQrqHIOIZrQa3zxMELelw0ewJECsy7dmgv8+R9KlrlgrReIaEzwLN9RGsM7WeIXHi+tsdbWn/xbRQkbJgMnEr7lpaVXUCMocFD5Lahf1dfQ9A54D021ZHZfDAkQdQUsRck/wxskdbgGZLeBkhEWMVnBNDJ7wQtknSZpEeEcksewDS06a7pBUyKPDc5yCqvQG2xfrjU4pbINuO1xdemZfysTxYW7tftGin9kSW53ROXeyCDdUfrBcqwk33TYK13kzI4dWSo+gGHgyAAk+axPi/0+zDJlgXltKQ4atLqQ/kK3NiyuGwhu5HrYG3yXs0Y4QXLo3dIExKtYQLKk+sSVI6BzJoI6QHHKOxCneOvd8ec5bVDdw3EhesomIO/yHCW8FovyZPUa2zI3dAq1pXM4Fpi7Yv+zLkKaCrIxB1m/E0YLqaOahgN17jn7fXtcBIsg7N47n+oakUbQRW5U5oZJupgTrR+8ogs8DTx3RwBTBWMCYh4zoqBObPn/DENt4BtWvyjXoFrojTsF24ItH77u6HM2vUDU6bUiRXPP4h2x/BzKdySFwzItCpj9oxygg48I8sgv4WN8GlEAJehDaSXJI2siAf2xKpYLBAt6v8XyMAIVFbWjr54HSgjAkr6xuu0tgMatoZ+ePnZFHrKyi+ZkJF1iDkpQ2fPzc6PBEl3UtND4fm2NoQ5Jstu5OGKBs73ry/1DdV4MhUt/QCmbyjGrv6WpYDmn7ZpsHs11fZ64y6vYtmkITNagTtglcptEhfLBCCt0dCS2nQWf90fMvjvR22dRYSjMf+DA6FL2euBoW+76fbUpDHybxp966OPQMGsOcIrHxQep0aoWy/vfXpl0sWrDApGEhQgOyx2prd+ecBSP1U53H33Ebp4h5JqrrCue/u0oavg7aNJ/AaOeHEtG5282H2D6/Yg+9o8zZmtZ7aK3P3+UurjVNLEY/CANpaB2SoB+f4A9FC7Xx5bIp9h6l+JIs+hBGr95VsajGGrocPC503We9ckS7GRGsU9J30O9a64rL9G/QRpGvpjVwRyESbmdiiDEUYHJF8b9MHm/MfeEXcNK+wyzXEskJ/oAxKczMYk1dFNZmocjlM9x9FYl0oHbluYXBInNnc+fbR+M3nVLDved6xq5BRwAS0a4nliDgoy99xHoMunsz9BXFetQocdLauIqDrFXCXTo4CCCMVQnCJ3bGFkLD8JDBK68ZRkr+U09QgjjWfQOHmbonBHBu9FCuLr/fwAfcy1Lb+6uRhm9rvPAw6U/CaufC+caARjY9qQ8HQWKyfsBL7B8S1fBlTSvQAxOYL+2bhARK2g5C9VqaaeTfuZRyi61EyZItyBRAEEwyMSI4v58JH8ldimuFborkccofHsv/JGFT/eLPNnPuzlX9SLyIAjFRNv+/E+N3H6QC24nqpIrxadPhc2LnuO9zAlxMbXUirmCP7k/1BqK1+o0t+z4nnBAKv5Cnv08mn0YPERre1O3lczasCVNqKve7K0a198qZIKZMFBtC9G8eDCjcZEgiovwJ2aZv79S/FA4MvRerUUzsJewuQ6UyYhhzwvl4I5DkRSQuawyzoqS6LHLOK2JG8FKHeW51d+FoGdnv0AYHaE999rgfNx+KeBdbKy/V5RzKxwoLfvI/hBLdgJ2Wps+O2vaEJUQf2idCTfSPELKrvLvzZqQ9swJDmfHp/J/Ptqkls+eAbpE1PJKWhP2Tb5crwz8kbJ65IljmLaeTrX0P28h++AZAZFg4h88ol9L+wv26u0gyZLPz0nQfW3mvayHzCT98qGd3Wxg5zNUEz9v0PN5Kkq/D+HM7GPpb6QN26NUfvGFS1ntFN4o/+JECo/rQaQof/O/r0jh+BYy5kB3/SoLS2XLvsxLxxleAToYiDQTBdJp46AUSyVv+xt5k7/wI4Z1MS1LpvQpA7fzZwUVTPVSA1VcYHw7eW+9xdKHRK96smiWTRH4sonVJJ/6tckTIN+j7Y4kptl9nWVGH33eOZFjP3yn+eOvl6qtNk/o+JL11XaR8+uw0ztWv8fA+XUOVr0UzbIhavuP3VkOdnCPWPhlahzlVO5YspifR7qkTaXZFGirjH9l5mHExz6qWtefB3rh/pEaa1MxrF5bxjxCGEG/oZ1eaIUk3hHBT2DUGv882ty2/CcKMtIgPChMp0bE0JSWN5RxWus2nSt99gSTqIsjZ2la4WAlmlAJlN+VbjCZ3W3yJ2MKz58qQrAonN8gXxd030tLDi3IDeLSNs2IoSV5PiOhM2DINwdFcWwgAONqRZEfRSFlx3a/drhrfyhaIWZN+Fw7NB8lsryazbVUVjY4ctggsTbtrFzjUSFvMBkdzrBO3B83jCdTb5B0cJQe/ISwEfwyisxa85EskGMB+7MVYyrs7LzcpWAKglMJj5SCePFZhJHm9Uf0oTqLzXBG1rySj7ugpUwk5Oc8VKrthHn+u9nQQ7V5qKRZN3Q6ZnUwFd7MCr1iIF60oR1PE0lQD7X9WQ6NEo0JDjd7XtWWCyYOxuWrcBONYL8EaYxUl4wS6gLSj/8WiUzmklXV2iz1t18rha9794r252gBt+arES599gjLLqpycuQ2ynR2yqqaW5HCPDn1j4wSHIPQ7VfPRrsg3dZ6zXw4q3UyhTddVdK6UVugrY0Zs3mWexXgLGHU6iz6uCVADiIPpF0cWpcqYj9bYksns85ftmHqeQrxoa9XVWObtj1zqpW7rb0Lb0tAUUTyOWZ7FXkHwo/64gqlHAryIvq6ngG6souBG9U6iLM/rRcyVutGjteb+4YPGNUHSSXwEl+e7ECsGsb1dVY5cJmkfF0xE2FXFYUAsCBvuRFVZpR70cpt2r5e1XaY7S5qO44T9I8RkYt+o8BkKCxjQ8Q9px6275PfUsGvo7U8mxvk7EmAxrmj4v6eF+wxUv1CBuPkZeHIqSGzQ+ZXVeP8ZhOzA+fYOjJkbfZNqUYkMHRkyNvsm1KMSGDoyZG32TalGJDB0ZVABonoCjGKr+wh+qLFuNpZCJ+JjCkuZ9Y0uY6/2WFMx8FRll4V/cpYNfUsHcyd+TP08qgI6J+BX2Z6275PfUvuJW/k1dNx6JJo7sw2Z6kQAtAcCNVoP7c/+0FCKrr4cj//ld+I0lp7GN/Rn8q/gM4h0YLsrNN9E7r9E7r9E7r9E7r9E7r9E7r+jcx97kRY2WMuLRfZr+6Dju1P/7U9t2z6fjxAAAE8MsxNlz/hCmlS2OPZ2L+IRWK/qEYF0hvMQRkX3PVBxnKNZgMI5ssFX8e720eZWtdoyCURX36/Mc6Ia9xICxo54HgHp8+J0QKuAhPeeeMTKcCIGBKJ8C3d3WCxXT/geH52IxC8fZ4vC9Kqn1pr4SmKojKmoBZVwTqKaNAvd9rGMGLvOeChYQnlW5IgCL3stPaWMi/gDFsOeCkeW5DXwjPYRHPmCfeDQ3jKg91ODK7fJ4DC/w9Zpfo8QOnhBVorTFT3Rwhy9a37LLoE4rudNBIZsSJ2QEkZGPxFDECl14d7CJW6dKjbQL6G9HKwyH4bZe6YTKcNMLCQ3IU5Gtt8S3OIxa3d6ur+FQLk+RUqGfnj9QaSGr05WK/jPXrQPSpldCFtfLb/Vs3B5rSJHWGHJ6zaLNDf321Xq7mmuDY+Us61iV/QtyDet9/pihWMyi0GSHudSpLLQIJlS+IKTVWK2KNDMlxCS7JLWR56Z/Lp7FQqHrmsHd2gv/bby3FxVpEhOyYickOGu5aE8dwbc8K8w0P2DMHi1TUDNGXWplg85ffp5KGF2vT2nv2YznOIWN3iyp0YS0MIUvANq5KX3jSxprVr1BHinA7krfUfNK4z7kKiC0ts4mQd6ODYT3V+QFwbdBlXgGmRTUTXbvCNlyu57p7sGC32ZFdBmmrYxwcR1YbQD+vMqatFAuXrn0i/w09a5eqA2l2tYBW4QBg62A0Iaj4UZTYbwYiVjepVN6Mqw11E/bIZmIyi3j7tTEUN4dmp9FnpKn6FbWnILFzjhpLlewNvG/+4Cef8J0iRXK+fnOBYkfGgFDIxLA864Jyx/f6RrfpREn4YPl/eBsI0VwR9rMMn4Df3ndIQQsPKEaFjpfPUA8Brq0QM2kQR77f/aowXu5B15cy57fnIUBuvV/NQNJ9rMR6OwR02oYObiKV5UmpkKifOS5Df47o4k7xeQekfOF0gh1ofqs2Gje3nresTmLtcV3+MZ222+1dSaYFpvAOqk/6vG5LtmXkPpznvjJ93ceiDZCL/7jrByEy6shxEz4YKcpCjKimjoSROuX6xnFAAAuK2A4TlozDg1m4XWI1ptssuE1R3lB5VOoAqYRPF1wOGCGt0rIsT0d5H+aYqMo2cibtxzsMoEdGj84NiFa914hsT48I8OletdDd1DnMGX9iBhBY8Jp6b0mt2RyJvBML5LPHNh93Dh5GsREMY+lcs9dC/LjjmoOkjGLJbdfqlBvZWP5rp8pcJljE5N+05OP1SwIVPJplockgC4CbMrsso/nMSRBrhCXU3Pir4v1NkIXu7DOZHymIrgrKaAwGgE19wNxd0JHC4/QofXoTku2yqYAw4kjpnsMHlkVD+lf54n+2lUZjbs4TNv7wkG4zcEOVmcKI2XVHe4l+VSeJlEOkzba+LD+q6SvGQrRG5nql3hwu5AAXRvUBRRTge/G7XLc839K6eskuMNi0ZSpmpwQjX73eFvWHopCZrhpEoL+RmctxTZk+5nwchkNlVWKuTfOaqNlE59y+vHfHQcWRLYDrUbrkgIYQkjd82zUeWwwqkf9b19pPTVZIIRKOIlH3QF9Cg1JmLh0puYVufcpmru+gJMLkvi7KUIR3Dq6S4TZTY6tkSwPWXILkkk9WFXwi+Ta4h92ZlauFwxHM60Sos2YT/lXewFAjzD3O58rSSuzrA2orBFECXWD8FR7JnZM6CJc3CHnG/yCCmN9J3cuzZTF48RdCYtLxsMjOyuhA+MM3jpL9hVAM9LkSICn1I55dD3W5fLU1fjAran5vSBtI/LrtHW8+owtMvtGIsu53oslGz/SQJuoqtoZzEk7qCFqk9lQ5OoJ1neE0hPZMzl/p8+B9s452bSUInOn4uNBUfGqdU7cs/J9h8BCvi33h9K//YG8fwuZuLphyxOamkTyfZq75WUqlPI6uy1o1C1eJI3fGqwAYxzRPY+Aju63AqtWDWG1QNk5KAoLbfsPLRGK9EI8z8CJNpJ681YCicsn6P9LDD+WKiIeOCRIMswaxqo9gktp0D5oTQTsz+9G21ifF7HPcyZxkFef6VR2zABw0gzjG7Rxsvzphb+Jvwnw89edMISAsTUOetaRC44aCexxEEsu4Zgum7SWYpKuN/n8QhdEBK0SOrvCiLdp1578+OuZVeqnUgTlmpQwF/ekUXsQAS0Dgny8LN8nDR0JllstMebzaYPX0mB5XZ0JUbpE8U1NmpAhFN30wRQ/dHkvRslTo+52Qg4t4tSqyPdsAaEgWJAipXX+T78KVDsiEe/MhKqEzfbKZsi66/hC95Xdp0to0C4AD3iwxNJzCXK9vGmerNUd7MXVxi77ZwnYabR/UsYJoqCEgt6ghw1RnfoBsrBjosbKhQLqJGH5O6mJ+Ws7WSYc5t2pz0XPgS8hwuVAQu/gD3bMfdLiArmLWU377Q9b+PydzYyM/KPiwpTiSmw0XDdv6J4hegZCWsk/WeSqlmCOH83Ju283+uhX31U/vNhiPJ9dQ4q3hoF1381ubkuv+plz9FTr83UBhcqygymf7vHPPVG4qw6X4IogjBJSUVaBp7wPCpvAGTYUfZJ+k/Gk44nWyXSHxKwjYbHOiKscpWEu/+4/AMQhlATQzoFPEzbjHe2VKHvYfyI8ZxUj2Q7t850dAlThj2z8mqYXewk+v6ednhtWozru315aNkp1A3fHNSz65u//8okyn/8NzgInG66b1wVgxeSzqW9oT8k2gLRphLSTItCyXa83Dyafx8HQqBYwS3Cw2E0C/PCXAfxz0ZyxKicMHlVKYne49BawG1X+gQqoT+rUbKBDC5ywbYC887FNaAI5m2Arw9LrkxZ1L08oTFqSpKnLjGxzx0ohTfxowtk6dc6cy7oEa1drxhQW2uv8Yft7JDVt+dxTjSPE7aKHwyBXPvbgU3Yxo1vU0oxkBBJ8+59elkm+8wXLnmXELEHMqgNUMRnwiAxNBPjE3LwaNA41RHwBiEf8ealXo6MjMSKW4CBYrpliMV3llLqmEjd1RvjH/H+92wwdOeQ5dwADJmS0e2EsYvxvgdVpV+m5OuSkXIAGuQlmLKpWKSV9N9HUB2lMv+VXpiiHkEgQZtCvktY4sHoTTFvT3JaTINXuBADB+AADT6I3NOJ63OsVPIinK0wlbZYnS25TY+Mji+6atyKSIhnYA9Oz1GLVaYrpUePueT9qPxmhhoTzVljZXoZja8x57lEWSb2I4peMiZsZb+OQS4030zKAJipKM/OqZs1S+xF30bpKMxIYc8LD5bU3vyT0qE/OPOE0lallHaYl75XAF0bwH5q2Lz6GzJuFKkPgZ4Obd+dYLXhS4opBBx+OT8/0JqRphj5MqUa/DHl9wnUjPiSc4gMUCmk36LqtG7j3zqoyGDvILN031WsZ//QGtt7AosNR9B6mpVWHIrdQPK0OPs/Qvh3iDzfpKm4Goe9HmWdC94XSi/vs7izavJjIehdZG3OlWOqqLC4BUL+Ptg0hx2sYxuNtfF502E86kGt1l/HnWb8bcp7TQSzhSHqNT6+e/PbghjuSEzmlwRxmDuyHYXVwU2JCS2FjI7A/CBUqhrlC8uk+2jUlJ6IxIGsuAIaQH8jogBRLluOYtLI8T3/QohgTsYMu0sMMPCKmU6mFVguXU8HLTvPCzFFlgccSsy1JLhSUfxvbEl+KDorh+QYgqOTUG6RAtEz2Xuu5eeVTedpIjiOBUwTYma65eoPHwY6qoQIyGBIjDA1IYB9+lXfiOa5Cs2oMgcDyLxPGq0/egdFYKbs8oIZCIMqsmp+BtJ16T9enoQORwI/16i0NsSvvDShfsp9oRVPW/c2/PAKwkZOc+fbrpiAvjOa0eTJwPz4B8jcAXlWA3MuXZQzUACg0cPCZY6A9G8E85QDY/l7lY8cTXctJ1YbpPt8Qu1gaVeql+7IC9w2E6CqKuE5pfQPgAikv4EUxnx3X/zTB8h8MD0BIWzgMdD0V9FaHDaumYGyP7jXL97DdWu2A71K1IIngCBvD5erqy3GBjAKnZSgfrLguThFHbEoa7sHUQrDGZYihQfVSdnocbyMqK/2+gTp6urict9Z8lWiyyhVtkKaWHcrkZHAm+NWARuBD08wwsDKVjeBMs6O772UFCMgEbjeEdWd/zRabgBYZOIFBD4fje5O1RM0aYfDTPtIIk/wH3wj9Fxyc2ksO6TkGbFlvuddLoBr139lrenvXt4EOZyigaM2tpXPLnd1ZHV9HSeC0XfQHvcRbR0WGDDfmqMwULe6TaVplVEbKiokbSAQ0kyaAONzuCwkyb6zMcmiP8sI/96mR2EpSZ1x+Klz5CsMas9wAAbGrGCGkxf0nf0RFU5MZF7km/H//wajX1+RaOgPLv8mfxjbnigBYFXuU57k7UoCLQul64tu/u/Npx+9cr0LaE+rvPEVcnqMcNfZbKqUmlv+O+7KjEZ013zDnoMmjG7yyMssTXY91QbhBgnP96hfMRwUv14BUFyvPNGkCkkGAmwpyzhDh6qC9e8x52R4Qg7//bc/Dz/CJIOv3V11MU46g1f9n6xVT04MxRoB6mXIwclYfWBnsfQDPNNs/YDctD8sYQgsSRqXuND4svBul4ZPY2NwVVukbiDIHMUG8mlSJlHy1adCdaxiopP9PU7yb2KlovZEavjIxyt8nqbN3pSrJ63TZM5/+zuYu2YsdhIiAQI3cV43UsI5He4MEMjfNxDvlwjaXOZQ2t/X6JsscVkGFoUHHrVg90CkIU3DyxmRJDxJwXZPp9O0CZ8gS+qXSm4mFqXt4PRtmrq8mY4eiZWzP7JNLwQKRn5Q48j5b6nnYS06NL6dYPoYqJa6rfWT6SWs99J8m6R8b2f3vaE2uyjS95XWrhbcnUAoNMZk3prskyM/nxLAipeiAfRAl6JOxYOkoL55quVJZvYoeO+SrgEJhE3myJjl/nhWcLXrDVQHkTOuYhWntYgkUDvUAgQ4+JpvOu6bbA2zMQco8wDoz0Ne8sQm991bkNIkMAxutuOEiAdzlpWowDyZ7FOKSsqQ/k+2G3+JoC9CIYUqv8An6Z30XMMeeELWvtlGXbOQakL/tXKV7kiKgtDPioF3Jsl1hkENisK7TbsZphtIb7icGiCQ4mdfOKVKDr/joOcR3iwQVZXjSTMYb94Xz1Rqh5IcgVm9FAPxjbniq3fQ/iEpsD2r8o40GI5qPRHVzvBHRvpkpW4n8jqSWQvWbAa2EmTcAPMwBjI+O9CuoD6uvEZFFvyrlpp6FkuS+Fa3mGV+khQsF34CVWFzLp4qtQcCOfYOyFyQVVKYUMY2FM0ysRuv/7e6V/XUBNwvKu6L344bK5zNPqIBz7YrBwGC3+NXMM6KfI0ITOT5t9Yx34kJVH92Zkx8PEdA2nenPkUVgACv04KuExDIb+hvroT3Y6RMglgwPuPh8twfx0VSNzFtb+zJyCFifkPqiXNOqB5Nz377QYKITDtoNw+5faA7jr9uTieVyo8d1u0FAd8klvZvdqfIdip7Sd9PWP/kZQ+80CG+SksguTngA0RvY3slOzKxC9M0L+wuShJh8yfsActG5NcAOOyhbST41cnnh8gSrsIUte3nhNhNceGzb4/CNFT9TXF6MCWD3qzHArcPhAKwXS3nrHlWQbjmaxEgD/fA6XffAYoL034ROFuy/xYvu+76sXXChmGCXp9YYm3LrvNcW6n4DEDPlNtKzUiaT/jGEpfa9VN1FMYOgbgDOg7DPLFJDz1kqcrOLAzJ9Rc9yZYvISYBchQkXn1gJeYjdxo8EazxLiwVa7DGh6HMMX+V8QT6IyASowsPhxwi67Qs9Mb2G2fY6gbM+r9xnvi1lTSkYX7ibgXmN31CTQ85OljMQ8jq41sXB4jtHqg0zSQAvVVcz1RQ+ddL4cfXqtBb02x+1uN+fvSEv3XoIaNjm2zsmOEkLijPmTXlJNaaOK9s95RrOnlPOcWM6qqar9cyZxTSCzkRZuH6ae7zQefmUu/jdHeUDKXoknGy0ltDHxdYLfBtqcT8XdP5OJVXjFf4D5BCbpR5pIMb/jDQJAB1fDW520eDDkp+FOGnW0TbQOFKSXeOVlhJEtC8+3U0RJbodr14VrgYJp5rGhUPInBQVqvbCf9a/c8c29Ue9d8RRk0fJPUOSi+sFooAp6315gjg/CyUbuo3tnw7PuOoJGgO8NyfRqJCeeEZSCa2ce1gCxtRhaBOWe23QrDhJLqpWjRRNFufiEeOP0OcyqF25ai5BKf9duxcOCGgY1EChYBXsrIBynDVBBFv4CAOkREMB38+yJIEhk1p8NEsVWYixxZyUXiUjv3AiseQMCH+J4ONxy2tBmgs2tbysFnrSd84PjrixQKJY+R+CD3JYh3Xwbou+l9khNwmmCKNxFeEnHzrkMWX71QP+uWD5eDq9xb7r9VDhuHdGR3qChBY5tPL36IokpnhfJNf39LsG4RJzH4Uc7JDVZFIiXmbQJOBMMCDa6PlsnR8oAEaH9X3F7dGnDhdhuuDn+LB2mf7vK0L/sCKBF1MtU14CLcQhN2ZSc6+JRcAM3fnYfKdUTsIfOn6SsqLIO3bN8sUpVUiAgvAajnRGsRSlW19BqX5ySkXmi0wlaG0Ll9ZqQmlaKldnCNmE0fqujF2CMsWIAJ3ikFS9Yx+KIxncx0oqtgjsRoKTrIwdNThQKfLVac2bdQ9GJfmlj/yAzYk/y9yVCG6cLxAk+WDtjht5nultawJtyTj3t/W+qElhtLlBWjaiUSDANSIeCsVz7VKhykBOlt1+XVTp+gjYYRLlHVdNNmW2n81+Eft7sTAPXbIhwpkb4lAak54MFcZXiumjGcyIO91BE4hjbJsH+usUuk1TR6GCFgVt5gYwwhovXkhdl1UZHE0M+srci9/5KZAJTEoAFCWFtq/1SAK5mzqrzf4Y1Zce7Ivcf4/YE3cPaBZ+ZfSYmxYqALGnfVkZW2qcnwp34wZrniQk5YD5T+OwgoHcy0XGnYR2EEd+WNXbstsRO4OOuoi1Y/GHJLi/Z3Sav4OL+Dh/S/t5z9jPbxB93h1L61/TTha9VuT8NOGOZxFW9+tyVhidCkNI/uIkuAMnsSn6SthHTFdLz9i2iv6H/RZm6TNDOyOYYHpHNF2VWSeQ5HxwHDOlg37Dr+QxdBHtqae1o7yiRgAJwku1BYunu9SguUjMP7YHXnXuS/4DMm76f/JgkzbE/r9TZIIrHPR4gMwxVjkR3jyg22fOT5qCwBnc+6p8+V2VoX0fK1lINjFRrYCxeijjUT71mbcMfwjbEGRXP/+vw5/sgh3SlxjA9tQR9+xua/z7t7jmvkix7qfD2jFQehoryCacBEaVPczYdp1PY0HYpgxSVgkEo1+62HywNA5aIWypc7TIC+eZgATUficYAfIEonHQz0QLdq+cEuh1YNi06xEco2WolIoXr5T54c7Gf9BtmK4BfgPzmUfO0vnv3XfFsYoUEi3BhIU2ErEGe0sABmY+MGD45jXs6AG+yl+B7XRxtND2Eh7U7Gv4oEG7rpXhnMLmdVx25lx3OWpvnuWDeb3KZ9qskpnEMR7rgAAJP7oxx1Tv8yzMa8sdL7msarjB/QNqgtrd2TVit8uOrs5UxPh8yW9wm41jLYAMElOFC/Vju6nUIhh4o8QvmoH2elHpzPd1tRJvjU5k8VMZUEdlTXFsve7Do+av5uPZe1u4TFwJKr9DXq/X7AJ78Yzr5JVSAm5aCIhFx+r8igirqIG9p27Gd1n8iHNxoNRFQH79pUNTJ1ljq85QSdvHTj3es/JNGvCNMzv/q1z5BEJ01HVbDLTvRXFwCh+IAH2RAzzrL9Fa1ROxjIa9nFETOmHsfXQMv5T1jLuJQvCwrNO6k4Xtlz/n/eLOip3y4Ln72V9GmWu4YSwy96ym0dmVyRYsTU4JCbQUZtQAekXodhRTUxPEfbxBwB0ZSfKatDg4vTWFkVsGuGZdQx1qPTtrTgq8X+YIwMSWB5qC8RHfV2ACvyhgZyGVudNZZVDaSooD6CqvchoThc6QGODUKhNzD0ePN6e2kCd3S8yKc+tQGP13aW2yFQLx1FeWY7oJt2jdgZC5gwmOtftvUJrPFGnPv6dTblagRGBOH7esL1y8LxhaIHjZqHFKFCYfWykwLkeN9y/PGEgboy9lIE5W4EfmrdxH6zVr0s7Y+o9li5IS9c/GJjZBzVgxYhRAAFmpudHbtUGKi/IS+n6KqyzOhvm9i0fOW6Y4VRN94SsMBKVQoXTpNOdtL7TJKRBXgsNqXwlq4DcvmRjBuMqF/c/sGEtWo3C+8owSs1RcBOpgx2TIIAFeWJG4hpBak37cF+BxVo5Bcv6A6sdtsthdqcapBSE5wsC+p/UU82BaS+mNyAfvOEK8hnM2AsRzVpEU8rjAAGwtqjC0iFL4UAcm4VFYyIL/BE+cKbduMXOmrP8SqtdBa+jU5vx6n/Xu1eHZYq7pzHrWNu+CVn87XGEHwtu2LakE5myTM0i9SwQf7xc02gR1JorfZKJ/fwxDuz2zbuKKFCqighVioh9Ye/kFlQfPXIRIGSqcuDl14hUqR5D10R+FQVnDaJo3dSUEov0+R8buDSdScl4DM2j3QhK/nha9d+OWTFEIFxBAFfN8HUFFwT4I8uv7RfA4iYL/Ox8jvZmpJTK2loRT8IJxj+wI0Y3Wpav8j+bx4s21+s9BOMQLUxzUPEFOjkkbx+kwfirIwSS0fl3HOQfSqrKWcI0gVznXNuUvKVS6sNBh77qSKDq/qFoaYNAbF4HFI3R8FL+LcISdp6aYL8MRBhlPM1C2FX7A3/CHWtWeJTa/Mnd1BiXJ/VS06TwUtHDcnX+qqE0dKv4Nt/SElKRyBmd0XHp3aJQ1T2GS7CygXRX7/8ERrcFHNrzJ9ICVVkjyKOngZj/hSFpUAA6Y1UfraaKHNiEpGwk84KLaQxqDoN/lkQL5l7wI3pm66TijBNSMPuq3AAzizOsRWtGZMVI9Ei3eEbrLPhmKOuK/n7YhWf3CcWSIuhBwykLJogcN2uLBkxWMi+ZBOFO+TpIKkqPwpNlVRQ9GAZnSXajoOjs1WzKwBbckpjhM2CGBhJmDjSba/01F4mj5hEOZEjW9dlC2U6pHy9fNI1lI5hiZLeaAGocxPuVoq+iH2qHrCAVWBDhpuA2JjFl9AoHw3GTo5AcUeCdSoPMudev9xRIiJM6rLhei2aB+qUNMQvT/QjMMRTcF5NVNToI3agszj4jhYwH7kix7Dlf1TKGTWaEfzh7tJ9wFnxtBoZzDqbOT2pGXVANoBkCMysg9b2k/xBGUW8EfITKkvQZeeBM6qwg8YFT0emncmuEAGhvGE+aTexojpjlJtiVt3EZPERQB/7jNhY4AzxBc1qvEW99syJA997+bIwYUa7WAP2zhylD4A5TGr1GCqVfGKYgR/DidYyYlLAs6ZSzHVvrPZPE+Q+za8/38oCrhxUhBw6CCt2Gwtx3GS6ViQVwxselCgQdSZJP5HGFWyykDFXKmnG3yA2OxQSmlTPibw7bUjPPSQ2vZSbINZzoMnsFnhtRHnCoP5CGhZKPgT6uG0+Eld6qy5Zzr0XNQFL64C0N3bbaz1OpFF8d9KAcwNOjPUjpfwYanK0gxjqsQ5dPedda66wUIru4aocU6Qpt1fFDIG4TVfxfL0AxbmNw5P2ykn0pZhZn4IAsDYsiIYA26Ama5gAaX/mVCHrpUFZHBQpxTLDMEXn5YE0h4BoAkL2vlxj1HQ0WnwJGFx7LlDXOjq7US0akR0jfBLlwgkWz92dNEm07a/DOMQ6bfS7Nz4InxUcEpXqNuEMdG5l3B6vpyYlXcMGYfNpMkrzdkikaBRSyuh5TWIk0jxzh6Kvqt0XAVpQXkvLQFYnTsxmJxPuWSMvU7V0MZwH5TSVa9JNharLunYX1Y4tIjByWe0upTaALhFDGe2ywgA36qGaUtYVf2xqO+JMqVU17QFISnPsCKfP1fVY2bIQ92DNZdnZHhWLu0r7f8fD+tOrRolfPpD/JyyNunIpFGeuR5HsmuQX6roQWOOdxzIHrj5Ea+1flkPt2kd5ZW3JhvqiA9Dg9fOTnSzphV/XsQvmhEruvJGwjtr9XOoQgI7+T3CAZurkCkkoetUAIWn2EthwcCKQj0DdKtNlydOdHQtnDqDU1uf75QE1SbmP0n87yOigXQ6BI8/zAAaj0Fpzv7BUuBCdgMPWttmk4lnP63ffrNo9RIDgW1Fb8r8NjnVpD9vKaAH+r6H6JSXQcNv5xe/xyiU3KUltzrJ/ZYU3sJ8nVoP8YXiRmmBgwv0gQ0lgzhCEAHMtsw2cpoAFadgxm3kTQLybE5CGJ7zq33fIDOTQ1/TOEn4qrlLtH01kfXHRPfrXPRuQ8Hr/ccHBx28K7Gq54JmRzYXv7rB4R6q32cM/TlDAAPBd+3Lyoy6icfgUTbSo8DBgKE+EopDmA2ENCxbDjnDZktBY7rVv7JU98ICU97KODOZh9Lhu0j+4tlIJw3i+rfli76egzwgW1slAA/q3yUJUkfc1WoW9OfdBjvXBUF1/mXaG9MRJRA5WvoeGoiYjG0z/FEBRYqLDVIv3amiNb3y1mGGiI0PGIm8CNdeCXOdy3AV36Z75Yi/3Q2nIjS2f4knQ0UDUbJQAJahCHrTUT29KBVIR6iVj0C5Rtsd3lGrMSQ7vvNvMgEE08ZK4Fq3VoRL+Wev0rkyeD7vqaVwQ+3yiX2oa8+c8HM28U4W+BYyS6iK/LcWWA/1+QgC7MaAJ2CAzbVJX4vVKOBe7BlZ/UehwAcr0dA2he5lTeZuutmk7CA1H1IUsP1lo4SelV3o9hHniSSCLfHUl+0W7KvhMn3BIkvGT7asgjqRH3xpG12pY6wID6yxhPtMyU+Rj7AZG9mUAknC5h9uuSEiGnJf3DVzAue0EG8Pj42eJ0v5TPhdvGYDFGB/haA6zhc3zalJ3MEAC99n3BqRyuUQI1B7PufGRINfgcVL48HP/MIZjy3Lb7epH70A8xyTRhDJAltJlV+ZYTWNLbXie3mFVQWxLM+JM9Nlf2OkJ2QDxHo25crS+8hdP2RIO7ywMKMfhR3yX3CGj9FOzulvOcCZwmcJm6zjSHNI1aXIrh+2gAOrr9PuycBE7/4GNfzieaiZFfKgbh4UI9zS/Y1x6MbRQ7twYWVtpcDHfAKUMljjaDqEVe7WjUMGzlQQTMp2+VQjJTopEvLjMs8kgrvB1IfHfWw+lZ5S9ANFmcZG9z4KBLe4vfzzWT84eePjxyV13cQIAEThoyu0HZa63NcmSLas1jnaWpvUHqijNxgvHMyoJMEeYzuyYAwnMULGgb33Y0LELb6CGH+99F7sAYHBmsxXGYgeSSdZ7FeU+CXpKjg/XN1V6lXAvzDr3opoLjuIH0bzQvc4feHM643AJcch+Xs1SHvfLN4DyRh8z8Q2lwgW+8CMwACUv/V1Q1sTGE509lGXDUfsCHWhk3k4A5AUEN95htsjDiNGmvRtIo7V0buB0zrCUdbaFZip2by1oVwCRQoa85faBxabVceZTaBwGhA6+omLVBaBr9rpySgyIPvJzzDWXiDylrayhQc3GQ0eQH7N5bTqcg3GvDLig3n7kL/3zDtrUIjML2WGDBiSUbQCQJEs6q8s9oQ2aqcI2lur6fJS/ZCGAh4kNUFrLNrSID29KpYnHkAFmyYf7g67zcnjHTdpNJWiIA9o/HOtaUVTKDzbykLzXWVMd+0K7Vc7EzyG+3cI4N22GH0yGOl5/gBtTVlK/6tM1E/RjfJD0PDds/ekLVqdrwfnC/vX/A0gvaF/dY+zl0FJ3/hys673SfxLXO98q5qy6bPraKF9uLEEfCfPd8YM45+PQ3rjzRUG5BxtcOlk9ObKNKTTF4U7PWUBk8ZyzcKly/5Qa0YT86VebwR/yRFyGl1Hc4gvRRkWCENnUQC/4ht3IJSN/v9r+P9eiq/OtN5v8KQtzNWYic6wcDWZP7x4zrxhBRC9YZi82vdToHSAL97VyUMNEv0O116QFO9cEyzHjkn8Zh+PTck7/DwGwSGpTN6hwoi+Lm5lTAq2RLckPyUD0gVbirqdKnaQMoaBC/75xlhn9DfsuLME7AOw/ko4dmaVLQEjs4E7F4lh2OaoDXcAAsbvLpfJirknSb8/oo8anMTjsZ1u6u3FXhXwHWLYmqD3En8PZwaSv2ayIAitZXG7sFYpaW/+o1meUi3nHPFp2xcMr6/qzUGdqitX4tSx/xVTXTE5h949BHX/6kuC4dFy6ypEEXwJAAENccAx/y6ZCPYl8ta5pU+B7wIXR9Xm0jslbdaGdL0fPwjb2YmmURIwLZgxdKaEX4OZL0y0NohRGgj/uxHRNGQ1yBHiBjzxwRhKVoLt/g4uEAVxF/Z6FwnOzEl6T42v8HBW6irBsG1aHHYK2p7DouTsPTpwAwFuvKR5Xrb05SLAFWMkDBRkt19X1S40ndrwGuQnSqhhJ5kngyz+5GzMBmCWi6Tbv+Dek0TuuVAbnbGxRYSxfJjf9mC3QOrpcHUGNy4S8BhiAegpLWrt7Fq9XhT5NVrvDO0P2gq+2xxG3GrUc6tSwxU377kqmUkbDW16Zl6mbid2yWoHXy5WR3LJrgK4V0Ak5giI0CybGY0QhACEtiNVpJQ2CrTg9XoBld2YRmTALtY8q5IY+eo4c8g6qlK2nEJqtbCxsyJ7EI8Y6oooSmNBHaWROjHaeiQwJvu/yGlVsOKKOR2rNr0wP37H/8EJPHPZoSRB1WujsEJ+kVzJtgG5haQEqWBPJbpZRKYOFQ0u3X1GHykHlZCJHoTyh8jT2leu4s9WNRrriy1lURuaYwODns1aaV6Fd1UWdNWgfx2ai+1D399XHtj7/drSRPgZGZa4CXFNMN99OagYmtsHfv+WhjKdrFT14CTq6lCACP2c7Co6/4LbooY9pAtoAsa+9e7nO/Ijmo9EcM9ACpQ8NF3oqlOxj9PNtXeTu8pkGvjO+KegL9mohTaExh6JKQWIojggYjmo7kX1JY6QVTk3uA9gfglgy41mXqFkFe13Af/mhXcImqnJ0UAB8LC/zLd9tun+/jZtMESfvvRH/6DXwx/EvJ7rceFmCnAUz+TGi7ab4AHk3+R5UcWt98b7dTYceRXWqIzxXa7q37AktRbdYTvVQyfNEnz66nmV8220LFx321E39f/xP4ZgZAp+Vt33by9Po9zK1MystY3vJm8/iwFwDL29vfQloVwHrIhYnMKwmLYfT7UARri8751Ek3dTgajyDbN62PiE/57fsMU50/1LHO+VkFTT2gt/GftCf49+M7DmZnbKSvXKrscrEEkCRDQ9eGVd/KOatet1PeapGzvSF2fcMck2Qdx3PdgjOweRcpvnT3O6x+UnR5Pgo2gBjPmf6GfkXyTjlsPI8QJc+G1QpQth2R1QGcKhay9Hpj82LXd3xkw+41uCkmjPuO+nPqSrDnCBbz4xCf+QCRbS+VvtolQjiAXn73wpKobIPKVSRHzgEZ7T2h9J/o3dP8BImIm9onFda+JF6y9n7X8YV8Ank3f5cRj9dVMfHnP7P/bCqGip3RvRGL/9o2ChebcYkk4ngJ70Ght9gPqJTaO/f4+puUD/cIygv9OG8Wb3QqVFgetCRxe5BlB/FZkgfS4F09L/qaGk/n+S9NO8qwQT6vIX0H9XpXm9UmIZnXbwZDoUDarBVfdaeuk4FjigOKq9AjMdLS3qskQNe0szKY5Ow1dc2E/NmrtN+mhf/MDQLdtLaRqKuKPNhKeJ+ONDYoiu0x1p+QPsPDgz0FlkzKfepExR9lyq9+QzP0aQ3hfgaYXdFw8g5lzOWEZJg52iQ+JFYQTH1AH5ipTgwzXaSML4FGl9KBJvZ7WoPrCZ9mQMVCoLDV7xypoTsA2QuMYqFsMcy5IzT2O4Cngb/hj5GyD3uoywkLm1OAMdpnvz0k2vThv8RX6mbGSJX9TNjFNYAAIBhGyVU5/xBynf/fmpzR1BrHyD6oCmYkP/vUPL8ktDG+hbFFiM/hp/E7WvznYcJ+X8nl7nA0XOpMoozmu93rQsLzoKRJxzW2PufoBFwMfMlzxyEOiPH2X8osAtmjWTwLhoLtko6hADdwJfK5X06NJKhvs8prtLHLirFY/ySNDvxWHX1893HQ4MNJD0jWVC657j7ypST6vLBShE5Ub1Q363gKvelniMMbfhnPuJQWX8OlHFLVBzDLIoVq3rkMH9UuwS1FCqwiTeHwW+pXUbS2145JW+L5nb6dHdL7E0GhB8DD4sb9ph0ciyVWMVldN0+aHCWmJJXKMsU0lh4osshE29NuO9+RTMO48yVimKQUdU33zX+6noOOjNlwEhp4HdJFFMj5KIEQUV9jBFtRY9TPT8otr1NeCM5360D1AiOXzmZ6rmIGB2CJLRCzxYLFIRLs5vpv++N28WKtwvhL348Th60dGrA30UlpmqIV06LQIfl3NnyUyS9AKci38X4NknCKKF5mourHT/BH44smwR4ckyUlYXz6NFOfeHjrLdYpfWUKZrr6w1iYQugwxK24zMzmE6zqmHWwNgCOErgLV3U8QdYoXFkWD6+XS5jPdba5PyWjqNAQCAAJZwGGR5OnDo8837rEBuAAglD2PPcYa1LTnWcQ2EQk+yHPpqeIhm2rYfD/+kHtcjKwY0NtubWD8RWan1y6G8pAmgnQ02qaRBTPW1aIKVFE5+ypHBY+nKazhtR4Nw1tLTT8YV5+f4Po4yt60rDO8yliwGfOAAIXhgABB2AAAAAAAAAAAAAAA==</v>
+      </c>
+      <c r="D3">
+        <v>1775191940125</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>banner-women-1775191956865-0</v>
+      </c>
+      <c r="B4" t="str">
+        <v>women</v>
+      </c>
+      <c r="C4" t="str">
+        <v>data:image/webp;base64,UklGRghQAABXRUJQVlA4WAoAAAAgAAAAjAIAuwIASUNDUMgBAAAAAAHIAAAAAAQwAABtbnRyUkdCIFhZWiAH4AABAAEAAAAAAABhY3NwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAQAA9tYAAQAAAADTLQAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAlkZXNjAAAA8AAAACRyWFlaAAABFAAAABRnWFlaAAABKAAAABRiWFlaAAABPAAAABR3dHB0AAABUAAAABRyVFJDAAABZAAAAChnVFJDAAABZAAAAChiVFJDAAABZAAAAChjcHJ0AAABjAAAADxtbHVjAAAAAAAAAAEAAAAMZW5VUwAAAAgAAAAcAHMAUgBHAEJYWVogAAAAAAAAb6IAADj1AAADkFhZWiAAAAAAAABimQAAt4UAABjaWFlaIAAAAAAAACSgAAAPhAAAts9YWVogAAAAAAAA9tYAAQAAAADTLXBhcmEAAAAAAAQAAAACZmYAAPKnAAANWQAAE9AAAApbAAAAAAAAAABtbHVjAAAAAAAAAAEAAAAMZW5VUwAAACAAAAAcAEcAbwBvAGcAbABlACAASQBuAGMALgAgADIAMAAxADZWUDggGk4AANCUAZ0BKo0CvAI+kUadS6Wjoyej0yoA8BIJZ27hdDJqsruCjtXXeN5iXH/l99akyeZ8v/i16yfTT/VfUT/sP9l6ifmQ/aD9hfd4/Lf4C/3j1B/51/zvXB9aT0Jf2g9Of93fiF/vP/L/dT22NUt9Yf6j0peTv7L+8fjz6X+ZH37/Ffuz7FWWftC1OPn35M/jf4r2l/2vhj86NRT82/qn+69UKHS4g9+/w/mzfbefn2z/6P3K/YP/Pf7t6h/9nxsfW/YI/pv+R/8P+X94D/X/+3ns+xfYQ/YzrgekAQCT1y0xn2ZZ2eS599SNyLlIoZvJc++pG5FykUM3VftcE3IUzMzMrABQXEbFKK2gJ8hX/FmUdMjCzXKP5jmjKz1Y0A8jvcMXKFm/R4/pXtCTzO9++3085nU7S4nDeRB0ItN05C6Nk66dNyEqxSMUBtfwa1ELRCjmGr1o9tIyhcDOifNFXw2ZaGXF3jrcPHyiDvPIJzqOb3ve9D5IUzMzMzLEk57qqpwwOhKQbhyPdDactwWWbTpuCoUbX8k9dBMlSFp02/DWlJx00qVW7IBJCBaG35sgHUp4wrQm0+uFs6KGJST1zk2HQPyqqqpLIV2Rrm1UypFeuM6Irppq7o+X+9mTTH9uaVn56L5vc6oTtD3HrO01fyT1rcuHQPyqqqSyFdyutRlzhx21pBdzByy2bUSDE9NfIdA/Ereg2yddOmq4KiMGyghBuPJ133oTrn8NDUDa/knnPBzy6jb8WoG1/LDNr+RWHKZmZmZmWJQMHBsoIQbZOuowbJ1z+GhqBtfyTzng55dRt+LUDa/lhm1/IrDlMzMzMzLEq7xcGyghBtk66jBsnXP4aGoG1/JPOeSFQ6bk1p03IU0jTpuPyLrX8k9dBrgLT2ccWiN9SpRAuIKrg4dPLnXTpuTWnRHUjOpH3NdLxvOsX3uk6B+VVVVJJrh9TtippNChouXXEmwj9vC/xdmEGGx4qCHuuHQPy9db+gri0s0Y/UME+D3MHcNVp32rwXQPyqqqqkl2Q4cG74wGgAKd+SflrJPXQdAetPcEhmbwx4ihr39JPXQbZOstLvZo5TSNOm5CmkadQMNWwDa/knroJkxAAa62GtQNr+SszX8k0i64dA/KqqSyFwxrUDqc2oG1/nANr9/skKZmZmZliVbgwUG35Gug2yghBtk49wUNQNr+SaSQGJRjtRg2Trp08uddOjPagbX8k9c5PEB5rUDqc2oG1/nANr9/skKZmZmZlh9PSMo/6MQGW9EP15ccv95+ttZyNvLRrZl9arnYh5QjwJpX6C1MjzLJhWGK6tHbG2IGQpDabtFe7cUoqqqqqqqpLIn/3UyqtYEeDeG/X8D8yTZGp9c3YEJCFwncwoIUR2tqCE/WgThPGolU87ZXSnHqpMx7IghjSWNcQS1bI4l1A/KqqqqSyF8uyTf/6HeQQ+ZpiJd86YK0BqMD8CXbRRj6245f4kjF5M7LHtCrKOTnqquDCq/Tn89gUwlWawsIVSDkcCvVTl0BTuWcZPXQbZOuft4UlB/SlBq6TYjh0jD+sFH2jB6cTlYGLUGyvtto+GRQ3eFEwuwlFyk42/Tx9OFynnzAUK253gy15I+szsfPjwrFrsnhz7ri4CFBol1W5WoNJyca/JQbZOunTcFVtiGeMhq+gEZSg/nj8nR8pYDHtAvy89d5Zy6kSJ7gEoJn2l6Edpd7/w6tA5j6O/xqhnHBF0f1fEqWwgrLbDx3nd0zcsi4T59P4C5kPNqLLObtA6UYqBS4dA/KqqpLIhu2bYdRwv6StFd4k/3UNNOkKFXR1QKiUFlia/zL3QijnxIPlbFrCTSJkTnReZec3H3xHkxeIy6TqKOeFdvotHdes03TWbJ/IrgNG65QojdEgsEcVf1q7LoGEpeIYwkODnTNVHJUSyQpmZmZmWFfoy0MXbwrh666UDtljlSIC10gAwWekNCwTjbZ3M9NeeQWjbbibY/yDQ/k41bhT9QGN/GoMTpk0lQJ9siYXFku9VEBuGfz4axbSsyLmaXC1smtLj48rzJicCvVVg2Y0gkJnRyjdl+eMTl+2Se2YzO4JNkjexKaUM9yIbNfyT10G1zFVbuMNMmTVxh8thQc1wbFnd466IIntQLO+8AaG1HVeauSYjBHZ5pS+/gngQR/Nb+6qzlC6jxCljNAnZkWmrQ0dOf1T5MUGGNFUsAOY+zyT+LenoZyQekNjQthtiMW+Wv6Y3wUI6AHq3EwwvVewMw0dcdsxSOciamYWdBB7ysOTNfyT10G1zE3zH/eJPk0T/Zj9BscM8IV3o2q2IoU/TnvMwpOB8r9zPihVhW1xlBsMvcWA+fcGr0jxt3gr+76hg1aDCWuLULc6L59L7XoziFYOjCSBkSootx4k70mz0e94TyOltIX5sGcOUhILDTnh5pYrX18ZWsAgEM3mjgV/Q2gttLGIL+j3uC9BlVCh/RJ1VVVVVVUkltkvjBXEzShID7P+k/ppbKZgbGhqN7+/fEN8U7dOSuKETv+wJSBegYHNKn8YCUNp8ApQEMHVziC5AcKfY7TIryV5onQ3OEko9aT0MUJrv8TORahtZLkPSgFI/nQGlmH2ZSxrw2zeif5RLL4yF0/cqQkHvEv5J66DbI18TqyXtCAaYfvEuNvwaImGcE042pRffW3/Okdy7oMqVFIMfFZP7fxKh2hffEWplhJyalp7EOsxQsI/vN1bGQcPQFbiA3QgZFvyliRmBFLYSoxcFVS6qJ9jsSNdBtk66bXDjTFoROZVA89l0K81wIU3O89aMeJp0w5fBQb016ssa0JmiEENCiMoatKvqj+rYFL/CApu3VFwVGsYH6NbDAYcT8v2shxwtJ+oJQknUfmej0SxjVOj7f8tyQFrpeR+GVDuXQbZOunRmANOSvXRpbWWePJTX1AV/khjmRN82/V3Zgd3cFGbPv6lLuVvJnFfkUdAmUqnur2yLyuXQW5z7G75cMrxUtCmoTe1drzAB3yTMuGpDvuCVs978cj+8sjRXdHG56tzXv+WkTGiXKvKQJr3O3RFWru9n4gzMzMzMzLCxLnpNoNQ55ZoM6+MYWXWK4nZuxNGPqomVjvPSdEeLMR0+DTQOrrZxYCexltP+YZasEHmXx3Psp1IblT9/XX4ywoHpIGrkPuoxHNau0B5+UUhSQ5Bhk4oyFCr+CWOXX2/YqVToSw0xU1Xicn5qzni1xuBLu08XWteR6oqY/XNlG1/JPXQTAXcvmCqTX523GPeK5HVgk0XRJromEn7XRJAb6fc+Qx92CU2AEYoe+sAb3jGx+ailhCUuRn0/52a/zfqEeymm6CFXpLWOsQWMzMzz4HskjfybDVLDLAHMk+Fwkle/OiQa8NlhALVwodpxbTPNFGAhbbFQhZzAaoCk+Wb+yrHyifKZmZmZmWFgKGiSaC9wJKTqQmzTESAf//5X4d0KqcfhT+5HK1wUClk0praNJNUbA/o244hPc8HE0Q0K7uLPR+teUoDVDurZD2H03hA4jj+/gw7MerofAe8H1jXvkvdGJB937IGac8T9m0bPo9yPsmgfBM35CRmSrCjLwC+6wnXTpuQpYV6Hwp8oCDVnDkD82Acnl0aDXrQcIJOWfBLin9ptYlFtGg5ig92qrOK/oIeXlvMDwdcSQf2VfZirOYkVHOrd5WApiBCoN0Z7ZJwKkEtQgMS0FUyv9nsMTlS68cyp4i25PjcmjKZvbBMTQISu7FLh0D8qqqkmAM3YiUqmg094t2RN4LW2kwDfNW7/e4wJdy4tCPHptgHg9yirw+rI7afVngTlfW2btCwlL18Ofg241dgAuI+KTQa+NK7Fo/Y9kfalTgdMhE5bm03AaxYeXaBbfnBOgoih79C+B1u7aUBSLFJyNs4ZiSiAzE4xSFMzMzMywrkeL0ErZW3fJJ9TV52SqbbjPt80pAzCmeqouTGkyCYNAEJlLk18j19QgdUPaf5k+p+ePz/kQDUO5a4Omtox1LJIV13rqTd6PKWkemzxz4yXbCupRI4PLXJVG/L1mzlKQPCDnXlfW4eFzahmoM5ItOx2T5kKZmZmZYWO01dNi6XiqAUD1MqjftDcddEgWH5k2hxCai0se6VL9D/gXkcso3eWdYeNrR1b1QFg4YZqDNfNa1NMUN2vDCTLM2B7bZRwjl/N2iLBNpjXS8Zue83ombXMARdcOgflVVJYrfGIAQGa0pGeeYVoxpwvX9hfBFDJbrMB1l357V15fwRmJiv91T3OqSAl4UQNrtln2ZGB7Z4OBoHJVSfuiFLmdw7nXTpuQpliSeN8aqtZ3zWhVISeNJSv4Yp5gvof21A2rCvkKZQAAA/v6fvfQ6ILUGFbQnM4F+BZKIoAZhMF76x1ij/aNZMdgirBKDyhu+Y9Ozo5UiucoAi4moznQv9Rj+zvKYrTj1X2r1bz8fq6hfkQLi/rSqE4pH9Kn0kylmIjfLpn6Pt4hQ5M4pIOJb5ESu1D/JctlN0jsPWmmwZ7/+zew2SbHI5c6HdBXL/D72v+X/jhD22v72oKYcE/TaW0PQDpqIQ1+jjOuKdtQicF+TSSzWlts7pswlt9epjl/a2yexnPetHfMuVuPN6mEOMRzs2+77+x6zTkPDCKFD/jzUAP5Vgg1BQksxFevLiZdHw0Aa3nOBomk6rNtOruM/z2Uy4zoqJxmGfP1bGSvW0ng0aEb1fc4AXhWeYnVbCFILUh7lR8ArCVhA0H4Y7xohYgOcOLkr3GU8933G+v55AhUXuf9HrVnop31+j1YWc685+aOiYdbIiD/iruy/5rAAoUleL6tLuzCK/3fMtzC+DdJPNpKtS1DrjF4JDuS/FDnGjDsyi/fez3QOl1MGF+9m/mR40xLpl68K6f1RYC90Dqc97Zsl9OP+Z1sTemvBKDoA/spcVm2sFccKdl610siKuZVVJChN/PqOMyTEraLh5c9Bx96au2FMOOtCV0QwpRnRfJNOV6ZvYu0rjYX9P37NXaUM02wAN+TFPKX7qW0LKA+yYKr/P5s6sc2lrSuAqwCp64E5u4oygraplCPxr3Y6oSpbBmrYEKjVsvqX1hCN5gCell6qHJ9qB54bGcDDLaCJTGXWZnKU5YmmX0X5DMXwtBTcd9fixFy5pXYkQEm93N23B40uJjMVqq4HZk2cR2AG7a5E9ipeOTHRTT8OKEee+OTyWPOROKYA/JW6pVvecrZ6fpjgbAzu+DZltKJf66FOtbjNL+EdFQvrBMvXXrnP+s0S+Xi0BU6rBGO8EvHEMWxr+je6G5fVJx7MTyqdxgPi2sCWnmm8a5sW4Fja15mIROe/eM/PEr8JKtWotLaLZ7E+hy8gUCK42/HA4AYDC/Tu1GCja2eT1jph0xXaBnNxF9iCveHyJWs2pnIevfrCjtOAAi34AHZWZYAuLPVbqhqzvXq9NWbYqps9wkq9bWcsqh3I+p2G+AAWMTp2vGlVX3W+FbVdI3jym4CzK2GXzdJn1YB1j072wMruuj5JwGdarhTQnPjeGSdJFc9yUFNrkw0vQkFyVbZd+KJEGMIhKyujwdBo7mBlHA+A5WfxE/DJvJpmzddE/nZyOOYk/r2gbi/5c6UqA5kUj3Ue7q4Zut3EGMk/a/laACl4/9TNIQmfv0RwTc7RsD//g9Pb/S3oGfcp/ysZmarHnPbvM5FeynoaGOhA16vS6T5c8Uz0J5lq9Ic6xQLcAx+DsZOGd5P2LUTQq8WfAfON5ysQK7nfA7Lu/NefcPX0JI65/zUtF8k3Sff+n+ZWaGb29H9zurfSGru929Dkf9FEGgqkjYmDAxwwasUIzyLgmygUY5MVeSkXd69HLaFE5WBT36AvYFAcsvHZhTiFL0q4K8L5LQjvHS1lkjMzf/BPGHIHRoEd0355mFHLbZrshcWThsfQf0lTI9YGc4Edf8Mu982IuKFi0yHMP0hWqMFvY5fp5YUrsAEPzachaZeHFvj2ozg5dbcw6MBf/8ZUP6F6Kp76UT8KPXuZj+ZhDiyRQoQD4KI+8J+R8phMvi5E27CpcyFJF6KIR11jF3Kq4yncV5GortC/XX5T1UsbJhVadUwnD1a2yMH7iYiC8eQQmGkRbhsuhXCpXqcbTj50T5A+a0IS9WWvC7LpKwjDGqnk/AVyFdldoo1Qu+A/VzIwU+8y/ngvFECUqG0gN0junTc96/N6CVgx1gx//ibxcpKwh+bP7wB9DOd1+idyrByJ6BRx99wd8YtyuV4zUb38C5DXGZoWrqDd8L8BfijPfr03eVJohpY0JaS3vo2FoBslWHoYBFPOUxC58WbYHUKqGOS0BkchJhxejqGRt28hngg2lwdG4OlBicsk4qP2leaYIUhQkLtY5qVf7wkfKUq2vihR6OcQC4MyABrLAlrSpnzgAABXaAAAMlIAAEysAAFcIScAAANpIAADRPUdnpryKjCOwUUk1Nu6x52ILZ4RgXeIvWXUEESqR1RKe3k6I4abNQdi0dsZjar9bO3Jxa+QS+F5OXuN9A/8QEnXEdbrwvI9vmlqOKghutg7z+9vnRAgO13mWcDqRSY0rlBA1w2GZ61F3gwC16Mm6/2oE8+4rnZT+SbOMZxJw+IAw6NOV7qV+enAHLmVKGKgnSwtm1cSEWAJWIa7BfO20r19+Ms+S9s8GyTDvWKhDfPdXCSqnnKLVlkBfaPpfGmgm63g4EiD71f4Tk36fEw9775CxQgjaUhhEQAYYJ6Npc3NEJG5t79SeKh4Hww4Mwg90+vIN0p7e1cECeAtsSjjJvUK0N8PaJEZ/JYwkVVyUSg0URI/+Aqi45YDrV3qnRsVTLcwYju1dpPqO+gktXVaIE65UauiirEwczsxD94yTpymV81O4WZjQzhV+Whtcf2CzQBYeYl5EShsbsS2ssS2xE2IdL4nIh7KBd051aTGTqDrmUazVcrJ00wrc4slFNvU5Iww9UcfOfT7aYjlZ7h9Jvw9XNBDCk+n7kgwnr+X25h/FJdZmIyNvJ4i6V2fnLUNebKm6YBPyTAZlz/QDIcRevG/SGUvL+UZKtESM7+bH5Du2IuW8tEYQPHG+GUALrqHpf2KU535hBluhJf82fnGcuX2O4Htp+h4eWB4hVmfHNZyd4kwDAAPpX4wjpJ79AeUEHv6c1epTqH0qX9zcATgvc/3xgmgqpTOq1UNieVvAOTxA7o2bw/oLkwfucMp+pr2QACWR3bAO/LbJmjePfPZL8FBcspxlR1jKPKZUz1zUx7k7/TvxFMQ0dtMDzUjMfFOuK3UCM8oEPRJnFk0m/nXcLiJDt4E5h0NfALEwNd7AO6SsEwVuQT937vkCs8BpeTwL1VzPraeedczfzyNdG06F1gN0tMertdZ34eV+fKaeE2yIXzHWzVGP44ZZDD/jMv+G47O+XfKw7Lgb/ljlIP91kLA24iICDvIA0PcUe5KWuQsACTEEJMruvckIlM9cfTq3Hzu4y/Hj8RauZf+wiqpp2edD3Hw4YLO3mMth+tzhAETr1i2u3nVzf3uqrXwgxUopxaOuhAPRRPdXG3gAAAzSuQAAAiSwAAAAhzzQAAAYmLQAAAXF7kAAAIOjbth/lieWq0ySOd+LDhaZE0673fOTLGD1Jk8pYvdZ3OZUe/TcZcxbyUIWfuqOX/98JoKhzmvHm6adfmdYVcERx9q+G9ivkpZ2IHcsNaWcmzCiHPKUXiAyRVdb9M5AZmQuz0QoHTiXe5X6pl+dTKY1TsPUerynI86P78FYc1LOd8B7vqxKHPUYy/kpp852gnfiHgc02yUrslzKZjEz4tLPbK+a9jPlzNziXrGHYLYv/S5rWLCQO8XAHydhI8FTvwnG8zn12IumcnL/Vyp05U2g5QQw+Z0UFTXGmdR5vl8kgoYEOYNd88lDlGu7UZuv2c5FYaee7uivSXdtUyGF3IMTdn0gMRJBKFq4Ow8ZXIBGfu4Rgxc0gPai1GjCRdRjOdBxMstecKQtR3fEuVa0P1jJHtvwuGhg2ioE1gTtg8kDuzlXvOEOD7ZfF9jUcN5sXuTItfz5pF/IQTsFDWslIzFEHquWucWb7Z3E5PZ3LpNvwViC2hyj07eVYSbhgH7cEL6JWR6Iox10ILpPVfK6gfSEkY1vVOU1F+CRo56pKpolWphld/16UkWpPVULdYcRxpL/O6Bn5cRqHXpFaYhMSzAzm5IWb2Z4Qm6JYbgnspqD6vIBas/yVbLoYj9vO6IAbGMdc1jObpBLc5arPnv4DgbCyaXyQEQAAPEJzK5bqItyJHf/QiLthYy+sK4nH8AACqwB+fs+v8PiX1181A0GSEbMsl+/xUt6eov+7ZT5JRRhKd4ZKvE5IynRtvZiEBvcxQlgz1lvx+pSw67ECd/p9CnMDOxNqt50IJKDfNUltoVfz4xMUOsZM1yIy+kd3/e0+CMj16xC+FvIfI6o1UHlGxq/5UceGCRPxJA5aANhlEnmhk0XtI+PK8rDdc3akFFbagj0rTX+e8pb/WliZSavY/muFrcDwAuE3vUiZF0rmknJ/7+bU7eRHX6FJTnYLOjUb/ys3sZ5uuVPs+TNWMq6cE6o/bI1KZkd92zbpuVyVvc0FFEedcH+kwNfXuE4FsqxzrCuXGcqPJO81TdH7AMsrs8yCB5SE2XMObuw5fDz9cefVneKrUvN7Sg0MAm2lpPBrSMfgRxZ9twqApEsVoEQ2hlACaCK+5ELD1xOFtZEgesFB8KIb0vGSqxaOTlUTnuLZDj8cuVDvAYmawzOPp54xgAQ44XpT1yRT2wPBP4LbV9j3uRfM4BfVoxhmdQPmnb6wbvbzl8WlGaVo5jgsAxI96Q0QFL/HlvcvfkrLlZO79f9t6VxRiWlkNSuOlNBZ/Lp4VX9WVPN1qp/xUOZ+YeQN9cYzG42JDiDe2mAuL3quoFUQCW891AOGepFgeJxRcxzIqgRky6t+apu1/a/HKtx350mWA+noh8yvAUwq9f2N4UN7H++cK1beje5VVPEiUJKY3ADKKj0GSSu9F0/wGeLE1Zi+JtzIQVAL6lJDA7avMICtipGkIZlGhXaHHXct0bW5zOnYdeceVVUE3WkCADwx7A0YT4ddrPhSBmOUTRULvi4BOxBstTbzANlySh4Q01hBtjBvr1StS6PYDI7MWspy0PU72d/WfuvW4LIytYW/U01S5Z7ATqm+HdSpMP7QDsPUODn3wGEJS1HD3ZZ0vknbFsoDH1k+N0sdTXMFPXmelnjeDRrb88PEHW86wd0gyntfOYM/NVwN6eoLC34ZPjxZD0cWWevBrguBKUhFWt9WBNtPzam/9ptJQXlfLfjQk+ZalIUVDJ3TiosWNpNDP+sLnMEJ/Hvv9/kDTjrS8Q0qZ6BEeF/8zFqfXuAowlXkhjOtbftmzg27TU2Et11SmhMpMyt8KLQvY0uDwpiaDL/4wysv2t01PmcS7Q+dPVfWZvPIhJO/MCWTT0DZamIFPli1t0lL+ORLoNBjIOzq0f/Yg5tggflIslztJXh7ZoMhYxqXx6VDro+Z4nXp3vRlXpaje9Eq1PfUJCL7V883e6DP7bm38gYG1kfprsiJr+X1LtFTIKqvBdNOYPee0WeKVe7N/ds/7rTlfItcqt+7ZfD1La9PLirAaf4adffnPimDpagx59URZOReKnAVekfEDisoZvgPNFCtmhO5x31lzcImMbCv8U/8lZ+WJPlrAR0mXWC2oheYtklQhgW5CTmQLvwXoYcr2H+ZEazN6+Nm6bBkCofrFGwnAcmI7FhYUtZdvGZCSz5lKhYwEZCoMFtF85TDDeU7cn4dkaa+TfpJ14wxGm5MrWF+zpD5H6RbZFp0qaaeuZjaV1CvGgIsHqKdXtuDzASOpvBEmZiMICSC+ss26ZcdXq3YA2mKYNiLCgbXTWn7B03p536/Xa+CuwPnKwQ/qNd9sQnJzD7ECsB2WXntQ7Hv+j3E2aPmVN73rRlbIfSGOZ4MR2+ip8NgVX0NGhF/gQeWj2qqL0jadZCNzUud6wTDtjj67RZqspKX/VkmMSUi0GM/K6hGQrPjI8hBYBblkb3LBx193Cxsrok3CA/HPvQDdGslpuNR51fHtjyKE/jbPwwguxX7XahLa45nwwNnM6um+ccL1e5dnYWdNCr5tz72r0vt+rKlKP0BC28LPVS7oOTr5jAWxXDCX6zKQg6bHWS/ri6wiXDTbLbsNqCfup5nn6bpFimRo+cgAsPZ54WhvdOMNl7Yaz6UzlJy0/Rx0KMDAddS2gsnR4cwcLPAmc/cV8ANQlgxXlOekEOfBnYamvmYYamx/p/cRMSkWkcdQLHTuMoKoCAYIlx1TljVlrPVuLIYHEJC7Doejnh+N0PcQVFZM13wWh7SNVUawkXPoIJKKFDhRqKF4PxSLFmXACNZQ7NBeTu3IWTTygXiY+x2/DxFKodPOGEYZ6AYnAAgwsIE3eCIIohbvlA6yzhrzboc1MXkFfiYIh7hnyYFU03QFaugtgpaHYGreQytIn/vyHDFyVKmZLSwh87FWv5Qcu/5yKCAy/QktFM4oDi7PU1lxVcKjcEeS1W9DqotscpiT9Ani48R6VGpynmue8hbVXNODr6kcuSSckrszHS1FFiMA7Lx2RlRO+UdBUCwLJNO8LpPCBneaFiccqaM4CW5kFbHriGrX+ngZsKttwEa2NmTynpFQRdJDbuXV7d9cblH5Ru6nCEKb0z9UMIaxSkWNz30GtfxWQv8wEK4zM/6HFX43GgP50LStfxqiXR/GuvoSBGPoCxjF8S/HMErNtwV8hWjR2hXU/LR/COcqwAT+afd0QZ4G/tvlguMxzKH2oL498xALMc3AmVJen9PgpwxDBMJJ77TeZ4//zl/JgElDUN0JvrDTkp3fLWodkJgoTjfftWCmZbRAiwJq5AxxJ+RI9PipEYjoZ3/w3pL3MBPWRNy3QzEQ0J+8jDcxJFhErAjSoqmCrPGTJEBdr1zev6CvydZBQG8YoEDDPUVSdWpGTXHP/M9BIpJpv30ZrMgSQeHmY9MBV3yiLJd7iwKLaQ8yScZ31VmBXzXXSkPVfGAfTImntLqFisW9iXTg+HVo7XP6SbW+iQsdGzV383cEz/cTj9fVlTTcxxkcFGw5M/d1VqcD8GwSfBGVQn0Rg618Y0Uh5aoUlyqDqyAfkrPLPf3Y5vO22BfhCasF54a6IN1v53u6hUdVDLKZCN9HimwL3iqTo5Vj5Pw2z6TS9Sps1Jpw91JJQ6NNY2xta/uukO1UdX9kHmgKdR2xRB1JuLrf9UYZFGmDeuI8O8BrnFLwClH7D5NMfC0EyjVZNrvuAOgy9Apkl8pXg5X+H2Kk1Spzxw3x2BeH88ps9AkVJjlnp6GNCldgMdn21DYO36BATlKRugnjGFLOdhwc9V4P0sPJC2MTNd0+IDNPvNyHXZQ8m6+crBANAvn2yS9HSJNZbOrsnPVbgkSyjQL9VDXb7niYXk9+Xe3PxsFjcA8CN9IZi7K6RXYz1sJRpxDL0HSGeNUPolwUGpRgQDd2hsUMLYgKr6V35yC9fdV9tnkeqKVqnHdeJp+nJSc2GafNmp4St3YNm7nKi3AFK+tW4w5/9tL3HmKTDL65oKcaqyL/Vr8Hx38G3BOX6VwhEtHVzu8VmNjbheG2AuWqnMHiSUgbUygt8IzOKty7lELjreuNl+0lzykn7gYDqDlp26Xc4/O/csB2PFfVN3bf85eGlgkPbEZkiDC1graWSZCBl6AxWZLqLTvRKVnMeSrEbQLnxms3vw98H67iD9pRJt9c1rTX1rIj8MyapLU6WnrrOp+jSntuQWk4+rptx7IXDEL5upuZ7MzFnwag0Gx/dQArASAC7wALRlQ2u42+suLB36Scam5cZzi7etHlbN5lsKNoM1sl4oYWzamPgOFLXj0VkQ2IAr+hujgFq9L/KXtNDCzk4/iOgpufzmPWQQ4O3StPze2bc4x6WldHfyBtsqdk7P1SGVCVifCecCf5ft/eAYC4khaDd075wRyzh+Yk3SQ9zVXozptIdJQlcQcqTvoiNvwJhsf0SnGEpvfJNiDfEs6SkzLPujFT7NBH8I7xJ5fUZloljSx0PktR/2sc/QVOknY0vq9T6r7z47ABHFuobRQ33+OAIOHRhCQnIS6nrlx9wcDiBYZHS7z/ulyN68oR/CVtKJFxiDTHAJyxqnZrYGBcyKmUFd3SxsMSCzPKU36AmOpAniYubOsed9ao6PWwXes1DtmunYlIgXZUZGPNrZE6Htu5HHhIXOoULzUKhkM8u2pxwXZy4cryQJ4ANv9dx4sOEMb0WOul3aRYpb4PXwGHRl646BWIDSI13gcVdyv411/5JHfMJL47lP6iiyP3NR+G4xnOdXhwco5eUsq6eM9dbdoC9GhNUpthuPRa2eV+9c6zQGYHKZkr4dgQT3i1Jd+eZ8rp2gMxP0yCq8xlVNqP8jr+8Amv43NOQ7bkwdEnFd8jUBMrLaRo3r4gX80xH1+q36OMeyzqb7f/F+BScMtzAghbwNzolFtc3M8Nw05Eg/8m6sBQpYyGEikjCV+XtMr9lgv5Kn4m3QLroom6H9HKlcq1gt4VltAcRZ7Pqld5vO/Sk4LIZ3JWGE9eE/2Ga4o22CFA7XzQtOlmdfW9p6KMOT+KiL3CtjRsRVfI97Em7hrfOUZdSvnzLquKFkaZjljGnLoTPz8qyhea1lT3yL+mU726+Dfbae8KlhxN5ZyyChWCtyH2ZRQy6UNb/7fn4PH7YPyoblZaEYVyqoosFzn4p6+ThjcdIFnvEHZAXQTehlujrp7XEj3Xpfxt7/iNVddS0rwir7cV+s4vss6UcSBURe9Y2gf33zKRF5ubvwKNNAHMmSJYgdvBo0P+D6BjJs7myt5n4wp6yE1kpGJxdqHnbAIDG4uG57BORUr3dM6s0ApSZhMrLKecozPwpbWzQVoNC4EVyx9EahztPV8rZDio6JU2mgkd9lx4LTz9tGBP/pzGOs0Raabv6xnaiba8z1EF+noGwgfr9XMl14h7JeY0opIUVD3Zanrvc2YeC1oNW4vNKLx3ykvLc09krH9sZyO270y6t76FsjqY50R4qXrOpwDZ4xwrmNSa3S9bjp0wk43c8z+CvLK3mqlidx1yE+cM+JQ+PwLFEKpR4yR8LXABLBXTpSQ24lDmcfpGcP1Osi6s/VdemHXEXpEIJfG/xw5YLqdRLkTzVyUgc2RNIIC9aXhog34kyMIINcSi+jrVMU0I8KQRg2EoWbD6YJXrJRnvWPAiBXIzlWol0JsjjyxY31BaYyhA1GSHcMPae6/jc+52HKVqMRDBdbaOKuZ77w6kisbVL8LpjGvb/s+Fq619KDR3DgFrAjOzkogbhvy0Pn5YXT+aYIC1AA445WttMlj1EkcoX0pAVIlDkyX+taZtS9HVnamO8K8NGmARpokXBmcP04isL7jjpH/FlNdvSUJk9WhU4rTa7HNf9aaes52ysl4EuWwYaPlRVzC0q27zdqKRJ2TgH9Yt2vo0zsPlJVw/VG4kxKB8plS6nEqx2hrIVGkF26NLRGeGsSrQjnrC1XXNRMZ1QINsAwgOUxYy3x7dHW05gFXQke6wUIfhi/g1IfZ+47mkyrho/SJzlV56EIwkcipJ+ZOOM72qnRckompH3Olg/mUmavR63xc6I7SsKtiYC9flT2pSNj2X5EWftFRnHjSRzA1Qg9mojdSmHJKUq3fVkueSArlTI44RYPvIro3XY0K6hVlNLjTEz9gaw8iedSFnml0gKXxtQhLySpZiv/BlPM8WyYRCuyWsrdkzmQtB/LtefKw3dBvHTVJ5FYl7L+G65efbW3ikhOph7uiM6g/VkCrfmZFnOgH40+2TG5oxUNjOuUk0WWkVFEOSdPzML66mrOzL4+YFEOHVFCYJYLier1N7WZNa9jaNDoTVmEb4hYaAs4NEoUqoFJsbH7dw1FcUxuvq7n3gKyVyVZkMRWS16cDGNgTBvcedr8wX6Qp53tEHAUZzIrsrujL0lsxVIADKHgHvFgSbHufvH6hlQo25nznqjS3JAYGpRFYzhhOlxn1Ok1OR0ZTJWN8h5u+/CZJtfUUn9nKVLa3ZOhr+0ZrgL9hTRbKop1be/Fa8yungJbO6WrJJdgQpygxj5iyUQCqF3GhYyf1VTFB3NCP8CWgfFKzO2SSA9gnaTHP2PNtggvQSE1Dh9CDsiyT45i8tNqvtwywLpKRT3fg7ncP5cMdEBBMn722pktkxPoJTagX4vfYN6Ue++TxmhGz8b0wJy9zoCpLZQFgMTamrbTq+PGEMpFMEt2F4tlplcrKKlbPaSe0s/kbL1iRHYmqyv7nRq2kAczDVvdQ2hgCGK3rpMl3xiuyw1lO85i0WusRqPaMBNNuKwZVR3zNBV/58iDBNdSGz9xt3KImqeneODwymNZy1dQ/AWGWuWERzjMfKcL3vt6L9t5wh7qyGM40F0gyPvIaoG9X1OuiQg0nyq3q8a4ME00kb5JXRd2rFrG5lUnnWhAemwYEFAEsvEUjPpW32lhxaO1pLndi8qyR4M80n7qqS4YxUDhZ00kO5438IomxssAmvGfB+6D6j8m6AD01Cj8AMvB2Nhy85dRv16Tm7yGxYfQfrfTdOhuU7jUUVxaBAspRQRFd86CnEreKXXAB6h2Pnfl7jtC4Px1K2hbwFh0mHFo6//kW1ggmhqPfC+jNrxCCECX9qTvglgvHNzIJAUjWqzLjNCokTMwuwfgr5lxbRVRn8vR5axlNOr1I5wFp3+/KiXpEbyyNLcU+rZStDAhuFIdeJLQ3Cx+7H6yGXuYH9W+WQCsZdH3NA+/+dbUMZJlVTu1+skNzCtZttGLbTSE2RBYn4U9lWODe46uJrjTRMWIdIyeFjSVIFI4VncgjsxMdtSk6TE1Zk8tRAjgmqLd8Wadjou6Rwlrok4fxEWdgfI67DnpOWJtf6zA6rc9bUu4cBJC61kIBm4EL90gS+CuD7Iy0IWXAEsf2my4jdbBOBnywwlwRT3XtXOkxO1AooHCw3UPqBULzlgMv6cizI8kxhXlt81nBkyVFxsPy/m/1H1aiV8nDKHgDAmwHmk0lGy8pdrk3uQowBU8trBvTn2NdQMYgXXKHMiTo2OnGpPvQu9aa/byk1NOpQYtL+r8kIPJcgBXyC0tDWN4XR76ur/xrAM7NZM2VaEx+DFoRGRORn7zIkrg8cwRDrJA1dGx1UddTqMZvJIKwGoBec8VqeQyYHBZnbCzm90AUUs3asY6r/7j64DrPqyjwQcja5gTgmyqBegpHCCT9l6MSenbwmbix42YESIhKUPHlL+nzybikjGPAkZPi+is+AxmAEN5mfMWj91MAEjanAbggtPXva5RFmE8VTpCd1Z19hIrCXEme7lp37RQ4s5iiU+eJhcaLeaHxxL31unLg4i6dHBnf/MwkIdngfD7IkG0uWBDbMjishVxUgn92o8d40f+AiX1UtwVFCvlP3FbaE4iIzsyqXcEXVrdsWPS7w1YjjnnLQuZOQMnFMYLsGAkCCswyYuLTx477qKugPF6m/j33KrKrPiYbNo56Y0mj01YuVCZfvG80715Jh5cRJob6PYdkAgWndI8egf7ZquTrRROlRSuO9kgqIIPIlrhiqYng8Zj8PvuZD21BFmrgXyrCJ4/+i7/J/WXtULr/nWZYTKPh2yGEgMPLuIukdwZzfbOUgh5M7yIPZH6zcftOjiVvev+awDBfJb81gGC9T/ejrqkkkMCR+AYMhQkhcxgLTPCfLUFmHEB8sfLhi12KT8bDJ0s6swnXwIlOPDuNwV1St1gQTTSFJnpNFMUNzG/NGSqD5MvjCyyiwtgk7NqZZWXy+EOoj2EWfkgavpr8yR0Olm0tW+dUdPy9c8jvTSpXIyeJsE1jhYdN6kHi5wmEO/lzKM2ZMgy+0jwf1iERkKbiRmdUCN5t4IoRMRfHaU0gbHmraOkbc5pfUUVevVNwhXAhdLkLmcVQwZJt4z3ccdIIvPkG0+yEPJ5C3jVMQOtWyLEfs7hOEcG+2Mrrgjoh2JwclhG4rXA+tJPHxXYUc/UGG9Ab6FlbjMM+MaGbjSBeAHue2gQXHNnbd7/FdlKuV5AxTlu1aSMSJbt7So7Ggq05uZb6svqQQ+/Vw3xyHVfIiRUM/BvZfAI+MCdxCoPtWrQY5ydeqqT1U69GQtNKi/lvLDbpzsgl2KSVDAIs2RKk6AEPdGinjdET63WEU+9a8dB8d4CCpR42J5kNMFRX7NKsvzEkhFxURfsj0KIdlTt5xTRbXln2AzWRgx9XivVJ4upnpqPE97Owz+o28IIQL7FxBUqaDkkPZNC2Ivi0XUpkDwb2/Esuh7Ogj80Csyo/PSnoU6QPz/yunped0jOXnU6sIdPvWi54NIej4daKPUrHn5Iyoo5jCs/21j6VdwE3XUNJnpHBx/NR/iPtHFHoQq8dN58OuUrFZ9iY7nhm9Wv3DhRiwsFV6k9yzJMxXyeTfjvXWPgMPGcGkW4oRC76mwfxh4JO46dbNKVYDfD5JbbEmACwbiXB1/tlGOaCFCs1xuqZaEunj5reJy2OYW69aZ3cjTmXFEUupVM06W8C1SEs8im9HAQW6nvUWWncbpbIPvjMCD7dmpI8lBaByiQNMvqKJVIYYTIkA9d/3rtjfEmJJVUVsHb5mb9CW0vrdkCKiHawnVWQhHxqYIfHcchYG+9E/hfMZlSqwgpNOzsxgYsCUV+v0df4VSB5XmPqhYk0gJpzn7Xs3DXBUdtRgqFuMygwG0a052p/exvo+Uw2lSjdrX/u5eT9Z32tnzXvs3nlJqoiDNxbr0dUqnczlFt3C377PDhtIDftO0U2kvALk9Hb6zo5ksQKNsD0T3mp3pDhs1Czixin+tAKJROJQjdnZbGlUBfj3EG9kBj2BnoqPbLuHMeVJzYPy/OIP3p8GiOcmRMayeV4i6GgSNWI5QI1V/daFqoFeJTOYMp/XZn3IAtFfVwFQienii7tA6nfoOkoC63WNfYrLnnoOY4OtiQR2iLbfcfj2nS7qAh1c3v/ixGJPgTwYi5IfjFuMpwWyDbcrb1x2FDxrzqFifoBRHRpT0JWxhwjV0gBiVmah63dbgQomc0D0DMucvDpwgFkN6QB03BZancUkNwq9Y5eZuII5G61cEW2/CpROGAKdsQ9SzVL/Yj4D5qOlxt10GuzaXuiVqMp8tfAISYRfHI6CEvj2KJYITw6iyJfwUK6TKXRzMFfWoX5qUjOlLLSqg9m3k+HCCxbt7y1PZDAakRhcyAAndNEQTngPHu5BPyk1ecnWRlZyF6RK0dANiVX5Ccwdi/6Ur3cJ6PBdFc+QldaHaOVJNTZQRlL8HX1xwpN6n9vwcA49nOdLYB/67X5q981gUfqnkwe5Oqn7VdHrD0q0HTwY8jHwkxJS1RfbsXGS6r3jICj6vj/Qd/sUIRdCcmzLowMeyoZU3VNsyjj6kWXEpUXkNIybJdX4n0mILqhG0G6jcfj68XhqeI1kmdcibYBiIXPbOTtir/57NU3MIAyXhV1BMVtNXBt6QtOuyLveYMp9gN5u/Yk6HISDgv5axCV6E4ufd15564uiU687+2j1BV++Xdt7KvzvRkOxS5fYuOSwIRcJD6Z1aUaWwAxBCWzWgC2GANCnYaTfHYcZhMgyp3S9PiSbza43cHjdQwJd/jgFaEAVU3DuwrsSkypl2gq8nlnqtf6YEmxBsr+b8OBZnd5sD70WAzh7HOm9MgK3FZOA0wBRUxbr1N6xss90y2nTlaVRIv7G27clgIFiyU+GgnVIn6n5CaPtbKuikkIVDe+o3I8fEPUlaEQYpGl5q3PKYmyybMTJkVPdMfj6MV9tQzd79b4zcIoImkslTHA+4rE/agDyh7bXPqKGC8NRutmlw5kWoZWU+7OerTgKK0GuG8e5NYQipKwH3LDtXinjFvTC/kOaQGxzmEACBSLOqBiFLVl51Sat9qTT/fpsonbV1yz0AUt/vzdEVFp4IyAC/OjnAoXZ09RJXJ8kmNF9ZNzFxBl2WS49eWwuZGhS+v1MaURpaBB3wLJyf1R6lZOsiik8DzhU3IE2I58q0TFNCYo+MBNlxloJbyieSefwynJWNL8DHSdUcd8sEQ0nn3OtovAbCa7ZsFd2ZcSKCK4NX6B1bAJmtYqpnIrxo3jARs+azhJrwe8wExlUsD6/Fxt+yUAap4ThiZ8U3wHBD1UcvgdH9VHbHqTW41nj2yEuK5jmXoFxJAVMyXdy7y6nQuhUuKsCHXUnDF8UQXTTH+d8VYehwe91EALCZVnG8iUqbrYFfAGZkWmziN6huVha9OSFEiOAUgyU2PBshwco5aoJrtO/hoP/V6GRk8UYkJ5dcwkKU8ImGmGsQOyyl0TKo1cM5qJRVGA3hsD92+SIei59DlA+kMCRKmwSeg4SmFk5OHrBwkOQz6+1WuJRRjYboXt8ORpY2yzr90cwXgh5TdVKiDfOSLdGYOG4iJxwhPZPHTpSI9vE4T336GeSn9wsBJa+jHyT/8ZJ4FKUg6KRkHQxGJqYtPKaGOpCrkC2ffFTxftIg7X47Qy7URsGMRVdwtErgTldbzLKtk0EkksCbM86Cg2tqHfWdhl/j/juO0HhjmZ71wr2vpPMCd+jEOqUXFzmX01/lqUIJDN13Ukyl7j7Y6n0cGMtZOvVp8XncRV19P3nbT2uMNRap5L7m3nFk0mOnekrV+FnOnRYb9i7WjX5L6xL6GIPkDd0OAwZOlSYIIfVV0NkaOqSDAry6Ebd3188n2IlEvURWk2On6J9RoFt32zB/xG8MVmDeQXkOjaelGgvIXNOHYoZeUD2ZYlZTo9fCI5FAKodhxdAJ9QVJHguY5+ss20nRqYL4mVsPPW77rRgfAgE0wprIZzXNjbKpxn4FuSCd652tf0Uuk+Ft+jI2aMjBcfuORqbwX/YIA0wAx7hPXeBhUkAZddEDG91ZIhqD/XLPRmJO9a3s2SglSPYyR9jua561WgrBtQcV8FE2qdtCJFHiRGxSXGyA1hpAmk11BKroozDzVDhW6DtEA+TPepNZaRyk+GB0Yb6fOqsKvgWW/OZxOjvz1IH+GcxvKwxj3qxJaLVm3uEqa62KntucYyxgS3ko3gteobTl5CxE1urRXs/eSrowu/MByDo6LHQhawVAigkxSEJ3tjKqkquqBQaYQUBVw7ylFZ5rLQzshm4oNpde6a/Iv5j0puj7rIYunPwOhbdq7Aeg1sL0dO5MLg7I3PGpWaR3DndngYBPKAoX59pVvQ6naILCPOvtYmmDqZh+Bge1woinYInFHitxN/WXyPvTKNygFpatCxJn4gPLqjyZZtB7+4+vpqMOaQwwAMApm+J4QrmI/83OljYTLXB72vXDhxXNXD/j1vzMdXqTc/ai8vhJkNNAQ2QPLsJO5/BKNDhGm8qRxLfVhAU0MUkAl0GghElbJn+56afRBoLZvG1NjGrX60nHgQ/loIfh0iUzr2r8edSFH5kPrT1AkAnMss1mEQaSsBcuJNYkPpxQoQNUqI9z1R88zLNL6yaOTXlRUn2qHQ+jjQllS8YbuKUtzIaR6glmrBHmolTmvYGFRw45ZIdk3phcLsJalimEdrF/YHsI2YzugwS4tJVZ61k7jaKY8KxZqU8Rjv+7X5c9Fnyzpkk2LZVXLid6bfVNPJaStvtstbU1HDHrUqTl+Z4XVKI7Cq80LK7KjcoPQ+CppokvKWtiNFQ8wlu3l2Yr32n1vvcVrKaXuCilKHp8qhb93ujtN5O+dRldkz2Jps08z5dHM3UPkLOIS+uM8MEReeOxJj+nbCle9mL9Cqq8SqvbentsSn1DvkSs/LCFnDR7mG77Eev51qCo5K7R3AsbN/iG6AItUG8vLy9G2n+aFY4zRBA0stDVZsevxOTOKk+XE0Xde6KV6z5Ra1EucH268Wsfu8iaCIHzhIjEbM5oL2JvTcVCcfmHYKaxdyG9rTSG147BlDIS5/TPRCF/YYWcyXFKBDGjl92VgK7Lm5LIWPWoKaYp4CIr8mglSGmHM0xGTyciHNVnpUjXeCrH/1ikqxhWyqy14t2olGinjj421LvMPBKCbHAuj/HYWNsrZGD4w61Ql+K+FVU6S5LH6M7nJElJwT7IOkhhpnhiQ3cRZ/zGUu2BaUItmr4ytX/L1Y/2pg09JPNvGaDO6sqI1CTj7U9y14PXyrdKeiu1eqdf/BOIl0tCUav+ihEnppjadR3ULZXlkwP/1RR0TasO2gRgg37bFqk8xQHsMK9EHvaKGu3e33b3YhB9eGhAYxznCrx3mMNqzfr9aK8oHGja81Ad7b+jwfLCKcWyr2h65E4WC0bxjO+ImzBN6TivcLhP/w0LDkUPUodFjkQ8VRWxWXHh3PdCcRbQvfBFCEjxL+F9ii6uEFsCWr1NKQkRh2fjfSzvoKp45G/8/MtmmjcIuai+N/+Gg6kdIjsfjoW5w7DmXwQxVRyPZYD3HEkvAYcNYxtSlhWnk71anUw/mIBCYEHkvMPgw3TzVOKYV2/oDqC5NoKaAfjY7kE1qg0Ypt/OLq1DAj5UmczcOH4Nu0XEheatz20ocoY59MNEDGUVoFtEhpOShQv7rnOGlx261uR671xFTgGKep3esdFzlzF6Fd8QcKoMzUpHb6jaFokVSW+5CsxAk7C5tmGed5R/5a/BnXo86Z573dfJ/KNdns+xiPwTEsEDuLzPqHjkQ9teLH8QdhMRIiWzWQYYT54a1s72gySVKcWzgSQp+sAqUuO8agEB7lJx468l26RAeE+7wxPTABVDCkZIo/iN/KxbOrF6uBAtHQcEwiPBTvxVT4KxjYavr/orN1O60MJepXOcuYmXVbC1WJAcbqdl5eEsSzUaJyLIfZY1rSORqMA2eOSQiedYIWwm9TJ5SDeD5w8xP4V1V6IT3FbwjdR5xAmt1H6cWqaAdWfTVlgsd8ewtUDZtdd2i4pOZtaUN7Q2gqC8+sy+NW5Z8XOOvNCrgwgb71iLtN1GRFW5sqY4zLRMgXqpUd6Boor3YTONkkQejhGqvnyZtuyRs2cR5MybYscPYHMsiXM2pMnIVvs26B0k2mZSvgnPd2eBgPz7Y1TxVc64XaAneS706pXcsIGIIPW2Lfuay4pDMUf9A2CX2iVNYca2Sxb6LfQxu4WRBAXPG6EAgwQetScok+eopkobF5HGl3KtHsmnLhluIXIzuFbdfLPukJSUzo04SomGgEfwopKQnCuzr2BTuJYfb7s9tW8CO0MJCdwdXKmNHp+Tma81819hqG85BfwlNLhLIpw0xEDqwB6RArUwax5la9na5qdBeeZNtBiZ2qJQwi7z0NDlYCsHzCvLYOiIxAguNWcl1nFTCC5t5rgVo6Gdf+EZWG6E1EdGaYXgtjD8EETs6haFp5RlvsnI5lY/gCh5zfmksp9QXlBzFoJY572PWrKsuX7l0MpbsnZ4NOjrUYDM4HVkLVIoElewERZt9VEqibc6wuIG6I8BzjVa5o7CxdOz62hAtoybzmDzLrKYL9iH4EEFIgOAdQKfoqG3AHYDy5DClK4j2AgnT+0xljEcxqrrwIEpnPeXJ2HXGqJ7E7YKIC24H87QJmrkiaPeC1rnJwNFzPQQN8pD8WcjnguA3FgM3Bl8Z9xzaI4I5y1isL4czl1kjzLlhac5AjC5KF7JaBE92MaJp6rVG7w0XaFUvzCDbYNH9kzuscdz2k37IBU3hJ5hGJqRUHMOeKfrT7NOaiZ93cMgb8wetd9vqptqJvtER1/AnET5zBy73l/n9MtZIZ/HDfxxAQBUFUrGzN03RVEnbFlb24JyR7LWJ3KVbPS4AMyda86W9t+cxgrZiUXgfEwA1Pmwxc3orH9y1ffLCRR5X8AHd4FUa3o5xE685wDv8+Vl0ibGgE5EKOmYNUfnP2apnV578R8/iOYkaOMgk52jTOp1oBhqGe2DFgk3MrG691y2GOr5rUsCY9fRqasElxfKusujIl7TMeQrOue6K2KWdOPPQALTgu5C1FO8sgX7luDZiZ7ISPMLtWxlFs5tfGbhGollN+V/9fp7bBF+vwC6O21dVho04trOJCIdZ/a14WqE1glQdngEVaS4vbpG00yMgwrViU/ChbyrdHUlPNMoQIDQAyjoTiNIMwQQMkX/tM1S15cQEZLqlxBlghNN/J6/3lvL6kyteP7X/l74kEJ2Bbjc300+Nb9ZbAdqizmv8cSXlQmX6K1dMOpykPyZa5OHMr2JgPl8doZfaSLq+TF5fgf0ZSjoirD1mI3o4YTZjtCNoGvBYv3ZRVdbuT2PyTSZ51X70va1gpGE4ED9infb0TSCbyLlLPZzNjRHa+4e+rj5JO5c43jTHTz524Yyx4awxxNY4VyU0PL6GduPhbJZ4MOdo8hZDsEnBsYX4e/BfXnSM8tx3giG+36vfCmZiE3YjXYzpBfJu5koWeW6ulnVNcDzxvLIGMMkd6Q9Los4aQD4A5DC6hCOBr0cZ56CqvXOopwAsQJnx3SR0mvUaIQV7PCKHTSiePjaDnx/6BfYC9LAldePAHL/wSJDYxigqgOXspg3fo0P1wL8G4gSQNpIYEilUFwi0MIYSXKU0qI1IjAXYK6F7ETgF7ZpSeKj3RnjiPIzgnP8nYmo+tOHSZcwFxUtXXTWypC+H12f6SgpB3ST7o5J2vvlS9X/A82X2poEzsUn0H4GnFciPRgxZ0AcqDAAX/AGaq4q2GvubaGMx2UAevqBWP3X8f8qW9BUqC1DOp8wBShYhoQya+KXseT+FJn1KI+ybKkpaMWsXaqHpuZFA8fBq3Q1/Va/6Y565bVjbjH0usoPOrkzxN9BuFmfBw58mHx7EVH3qcl+82X/lGzYookDPj3bk4omLKrC69/zJgOfJp0Iei7ZTiFGanhBd7as2UXsPT7VXzrPV6utD+4V+JwwNG3TQBqzsH83uV+1R7/Asjy7wWqU3ZVI6kywnKksVu5AuqiC/qf7yMhYk5VlwjpEzGTqP+wk0Bi1jGNlIDbjflvMfCGZ0tmDn9ms8FSq+xrKTreYuC+NipCQf1m3TMFfwSUwrbRjoDPQn1V8U60B87z8BEwd/1hks4Q4iYVoG7Fi1uyqNY6erOZ467jnI/2M14ROpddI+r2HE5BOIVd7v/F0Z13rUaI29JfqQrH4fo3qNE8pNqanIMJKsbjRdkCvLnSdFWud8lg3MygDaTVZokk8Dg/aPdQ7UQ3bZxKOcz4co1nVo8TlBZurbpqRJ00BmCZcWM95AuVlRZZB1DniskPmYDjs+KZhRghQhhets2Bckh4RtS7MeH70AwyTVryr5cGwxGVZTRafwkV/Ey6AO/xxc2cBP5wXN8QEFgZuUEpwKMFVjD8nV5YVUD0ujbaOpHXLNhyQawo3vhTrI1FEYHyfzJI1lAG3ulvFXMFHYYob8WrqaCyrcDhHeJb/wYRXmg56ap8Fs5/qNgCrL/vv3k3hUjYhvHodXzeIpJojz/JylvuRHZBWR/tQ3cPr8dQ6lCDLyuoVQtDFxTZ+vfqc1GerDc3dq1JIyPQEpE3lXDMhjiXOJnNPbHYrBbMf+OWLQeWv8JB1+Nn20Lt2O49mc0MRTOoml3DZPXqbwD/wh2u6zVL8TYcoHW9Nlv+o5ClyNzmOCqZKYZCHAhoKfyxqEIq7QK3Q+B4aDihfeQ/3642rcFfkPhHnMXH+XoNwy0P9tcxGmGKWJ6kwOpiE9HBWIi4AQ2Ri4IRqCRl660tEx9TUETv11ofDdbq7DzQ1gGskff0oVorYJGOeKtZEFmzChwXwWzGwU3+L1HR6+3g2ciSi11EPJTmXgiECAdoWBxiUPuHklfbE1YI0AKwFHZy5VHH0ALjhWf/fnV1Nfz9v1z8+9bIGMln+ZF5HAbqZBP+x9tQzG51s7AMimj+i9ZciKXhA99UN0YL4LsMhkFO9Dxlqs6tu4czEBfe0lmD1QZr6aRG/sZYgA10/hFg9Sb1COvigbYXDjS/yud1Yj6bn9zKC/fZ+tHfzUnFQ5qJnOl4rAOO1ftDw18DyyxfKYmu5EASoJXWXfPl+S0lLZRmX6I3sgQAN9aijOOF01mfSvNDutFHJyhiPpOzdTSBvl+AFp1DWhZBm6PcDM0MZ+1OPWTvgAPeuM9aGvOm1CX15cJul+/ml/cR9ihThziUozjUk5B1O1zoAoURVocVVDkL1Bqo4xt2QKOSpODNfNjMtVVuULw5N4NeYipptY+Ncnh3ZJM0IZBZLwchc0YOBYVFUNYynbAAf4afowaQDc9jLzu8Q5F0RDMm01MJjwUM6bZbAMOeI0z32m4l132I7bQgIaQjqtwvXDxzQ/ZKz/Nw2zMa8XQYC/upmKb4UV2A8oJFQUN5UT2EuDoYNgyHj41wZ27v9SosRki41cRyKmokyVqduE3b/0Bt1hmFlT5fNsDWEILlyV841vzXhlQyyd0eDNQRBRHfB9mr8y8ccXnRt5qPg8kNOtj/YSGimR7skyk8IPiuYAAXor2JzYZbId2wf/aQLYsbsnUOYUzmAna3oTcwTYr5cQkdF2+1goeCKliDhl4GtMlHbInh3ZssfvbGAPd433TLZQLqODpCkLao1PhlraO/f6Od83SJ1Rnrt8vctMu9iUz585eDszaHzrRu+n4rMk956Ouprn86mh+10kroD5W0VgJ5ZAIQzhDcN8+EGDFsW1Q/ib6FI99n9eMClIu/gUemvQVvKaulSsaL95Ug38pAS/d+po+q0isIF6iihrC0dd8xg7zMhT17fGuB2W3ZTdRnEO1DhQeg/TDVRbIh8j9OpoTk/X7Q3ulFrdZSVG/I1MiyJ3FUIVPryuNfMrLLNLwA2dOyO/7J+0zmZj2Y3jr18V7YTfuUVACgaRQtw01HqWzWU5hJ2ydrrBVsd4w8p8/kMULRw7/wzB2WPT8Lmak6xG3FWFdrjUT6Pvs0t7QAJwjt0J4srBDCQ8wBljaLrC0H2JUgP2PwQSh7tSJZHnQi3rpcoRbc0B/7VHnMLe4yX7t3Jokj0x/mg/sDe65+NrBpRVzhO1w9/KZ1AZJ+D5tHugFi/F4SHpbnXud29rD5E0SATyaPgmVcg+7BlIAEKq4O4mUbXN52A4Ic8ZKCV+1EzREgZMXGlnZICT4vE2gvOCJ6h+DOoJnfZWvoI4/jv3GYDLQEG4COI7M96m5bqcXE6mjqoPLhOERFVDoAZmuBE8VvPIflM4rwiugioaJEdJPBrsGChP7JDILwMydkgu201S3GUcsm9a7aQucV5wqhesL+ZomqE/0L/db6xis4b0xuZEz0OlYB1Leih691jdlR3lUWiDo1HYaZq0VEfnEwl3YxBXyt2n/4H2c2JPdNU+eUH795JLwxzyE2u7Z4J8SVnT4jkVG3PYQ/DsotxxvuTJNtTx1tehvYGXJQHjvuFY8W2l3aXc0fGlqLJWVgDuiZvx0ZPy2qwdRojiJKBmBBcfJt6OFtNO17ruMvycN8axlRlEI577EpqRt9zA7gO78G+NAZzoE+m95brn4m1Q/Cd1d7rSdMKEDjyXTht4qRSLVfLnFjNdM4NbFTKxWJRiyhOwhVm0G9jCWriTPEZk2TXPAKEjvUaS+2kj9A5DU+ISluD7Vc5c0QfJEmqKaZP7zinDEOvumjmLc31SZVOaBB49r4nJMNrlU/RQTYTLzwPAOcm0i+QDzvXD932As0iVkXnAS86QUTtl9N9hzFqOi7thf+sfAKT0MhuogCva0HY7tfftNwAAL/NhMwHaSS9+p6LFsDLFJ5+6JHqh1faByTwZR4urh7ltfROm7HUxTzZv/RATRrYTQJ4CYOulDqgoqidSe6nrrEy8IxRrjdo+PHtV9mAOr9NZW+Bruosxotz9mQONzEqHO7x5stIf0vAl9AwFrY6OVjXHdQrYEyFvPxx+j7mHK79sa3+UnXxiHkK9EDght1B+n19iXWy/63v6qO58Oack7EDUZKxuyGd0cap2l3JVIHrDk2UaoPJ5e9l48UZ+v1PjGuh4v53xBHuWo5zBvrMLZXLP2ONKBuwParm3sVlLE82/MQ7hT4/C+RJ3JnsKrko2xoS9ComRpxJ2GudTF1Yaz/c4hK6Wd/BRpuOibKyuxq2Nereot9eFZ/JoLnmKCN4UEDk2+NMHtOz/KTbaYLqN+/WImvCJViHF05VIh2nmWPiURiTRdzmpvUtA6eRBuGDYWLsFuJiy9TFJ6/gDsAuMbe6vMxS6JogdC9au9zDjEvL7XQfnYB92HE6QMt+0mgvTMf1WM8eRQW3yBtcSVlZroO20s8btx8uBntXOVhUJLim5KBaZqRIIn2K4Gax8ylVmkxrEp1W3f9zEluWUzOWU9I1iOeD1j4Se2IfoEon4lbr9lwlXyCx9Z3oHcn92mOPwNPuAWn7CDi1t9wyxvgvcgM4dS6vBUlIaDuSROGHVJ3JaqMlO9dvSXot9DSbflrZWLfv5UH+sVl7d25KXw020LlWqnxm1f0YGwj5r96McPNTu8qIYYhjlMhArhjUK7mor7QctnCbGyJmC7iLJYezapvKlw/+E+3nDRH4YFFtIeXgmLB43oLQexQvmCxJCo+TYgpjh2SXacLHDBNmlq1hoYHb7b9nh/2QKgCsb8Y69RTmr7gQ/0KzYzHn+bbWDhJZN+PYiIvlZRJuTGaQOWzqHPkKUPHZgCIAAABTHGkAGuNoKR889VOJpukJWmoHgyg+NjaOgGfQIAYk1fyrMXVH34RzYYqsf2C4Q1EVIMCbcVQcoXNZgY95lEC5GNq6HFXPFqkyScgAAAAA</v>
+      </c>
+      <c r="D4">
+        <v>1775191956865</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>